<commit_message>
#5 U1 Digikey Link added in BOM.
</commit_message>
<xml_diff>
--- a/Design Files/BOM/eSpark-BOM-BMS-v1.0.xlsx
+++ b/Design Files/BOM/eSpark-BOM-BMS-v1.0.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="232">
   <si>
     <t>Component list</t>
   </si>
@@ -713,6 +713,9 @@
   </si>
   <si>
     <t>C394024</t>
+  </si>
+  <si>
+    <t>Custom Supplier</t>
   </si>
 </sst>
 </file>
@@ -1368,6 +1371,54 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="24" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1399,54 +1450,6 @@
     <xf numFmtId="0" fontId="20" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1860,7 +1863,7 @@
     <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.7109375" customWidth="1"/>
     <col min="16" max="16" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="8.5703125" bestFit="1" customWidth="1"/>
@@ -1878,15 +1881,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="61"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="76"/>
+      <c r="M1" s="76"/>
+      <c r="N1" s="76"/>
+      <c r="O1" s="76"/>
+      <c r="P1" s="76"/>
+      <c r="Q1" s="76"/>
+      <c r="R1" s="76"/>
+      <c r="S1" s="77"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1936,7 +1939,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="62"/>
+      <c r="S3" s="78"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1961,7 +1964,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="63"/>
+      <c r="S4" s="79"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1986,7 +1989,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="63"/>
+      <c r="S5" s="79"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2007,7 +2010,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="63"/>
+      <c r="S6" s="79"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2028,7 +2031,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="63"/>
+      <c r="S7" s="79"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2049,7 +2052,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="63"/>
+      <c r="S8" s="79"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2151,7 +2154,7 @@
       <c r="N10" s="37">
         <v>10</v>
       </c>
-      <c r="O10" s="70" t="s">
+      <c r="O10" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P10" s="38">
@@ -2182,7 +2185,7 @@
       <c r="F11" s="51" t="s">
         <v>83</v>
       </c>
-      <c r="G11" s="71" t="s">
+      <c r="G11" s="61" t="s">
         <v>108</v>
       </c>
       <c r="H11" s="51" t="s">
@@ -2207,7 +2210,7 @@
       <c r="N11" s="51">
         <v>50</v>
       </c>
-      <c r="O11" s="72" t="s">
+      <c r="O11" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P11" s="52">
@@ -2263,7 +2266,7 @@
       <c r="N12" s="37">
         <v>100</v>
       </c>
-      <c r="O12" s="70" t="s">
+      <c r="O12" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P12" s="38">
@@ -2319,7 +2322,7 @@
       <c r="N13" s="51">
         <v>20</v>
       </c>
-      <c r="O13" s="72" t="s">
+      <c r="O13" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P13" s="52">
@@ -2375,7 +2378,7 @@
       <c r="N14" s="37">
         <v>50</v>
       </c>
-      <c r="O14" s="70" t="s">
+      <c r="O14" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P14" s="38">
@@ -2431,7 +2434,7 @@
       <c r="N15" s="51">
         <v>20</v>
       </c>
-      <c r="O15" s="72" t="s">
+      <c r="O15" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P15" s="52">
@@ -2487,7 +2490,7 @@
       <c r="N16" s="37">
         <v>100</v>
       </c>
-      <c r="O16" s="70" t="s">
+      <c r="O16" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P16" s="38">
@@ -2543,7 +2546,7 @@
       <c r="N17" s="51">
         <v>50</v>
       </c>
-      <c r="O17" s="72" t="s">
+      <c r="O17" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P17" s="52">
@@ -2599,7 +2602,7 @@
       <c r="N18" s="37">
         <v>20</v>
       </c>
-      <c r="O18" s="70" t="s">
+      <c r="O18" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P18" s="38">
@@ -2655,7 +2658,7 @@
       <c r="N19" s="51">
         <v>10</v>
       </c>
-      <c r="O19" s="72" t="s">
+      <c r="O19" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P19" s="52">
@@ -2711,7 +2714,7 @@
       <c r="N20" s="37">
         <v>50</v>
       </c>
-      <c r="O20" s="70" t="s">
+      <c r="O20" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P20" s="38">
@@ -2767,7 +2770,7 @@
       <c r="N21" s="51">
         <v>10</v>
       </c>
-      <c r="O21" s="72" t="s">
+      <c r="O21" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P21" s="52">
@@ -2823,7 +2826,7 @@
       <c r="N22" s="37">
         <v>10</v>
       </c>
-      <c r="O22" s="70" t="s">
+      <c r="O22" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P22" s="38">
@@ -2845,49 +2848,49 @@
       <c r="C23" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="D23" s="73" t="s">
+      <c r="D23" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="E23" s="73" t="s">
+      <c r="E23" s="63" t="s">
         <v>65</v>
       </c>
-      <c r="F23" s="73" t="s">
+      <c r="F23" s="63" t="s">
         <v>199</v>
       </c>
-      <c r="G23" s="73" t="s">
+      <c r="G23" s="63" t="s">
         <v>93</v>
       </c>
-      <c r="H23" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="I23" s="73"/>
-      <c r="J23" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="K23" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="L23" s="73">
+      <c r="H23" s="63" t="s">
+        <v>198</v>
+      </c>
+      <c r="I23" s="63"/>
+      <c r="J23" s="63" t="s">
+        <v>198</v>
+      </c>
+      <c r="K23" s="63" t="s">
+        <v>198</v>
+      </c>
+      <c r="L23" s="63">
         <v>6</v>
       </c>
-      <c r="M23" s="73">
+      <c r="M23" s="63">
         <f t="shared" ref="M23" si="13">L23*5</f>
         <v>30</v>
       </c>
-      <c r="N23" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="O23" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="P23" s="74" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q23" s="74" t="s">
-        <v>198</v>
-      </c>
-      <c r="R23" s="73"/>
-      <c r="S23" s="75"/>
+      <c r="N23" s="63" t="s">
+        <v>198</v>
+      </c>
+      <c r="O23" s="63" t="s">
+        <v>198</v>
+      </c>
+      <c r="P23" s="64" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q23" s="64" t="s">
+        <v>198</v>
+      </c>
+      <c r="R23" s="63"/>
+      <c r="S23" s="65"/>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
@@ -2907,7 +2910,7 @@
       <c r="F24" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="G24" s="79" t="s">
+      <c r="G24" s="69" t="s">
         <v>117</v>
       </c>
       <c r="H24" s="37" t="s">
@@ -2932,7 +2935,7 @@
       <c r="N24" s="37">
         <v>100</v>
       </c>
-      <c r="O24" s="70" t="s">
+      <c r="O24" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P24" s="38">
@@ -2954,51 +2957,51 @@
       <c r="C25" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="D25" s="73" t="s">
+      <c r="D25" s="63" t="s">
         <v>35</v>
       </c>
-      <c r="E25" s="73" t="s">
+      <c r="E25" s="63" t="s">
         <v>65</v>
       </c>
-      <c r="F25" s="73" t="s">
+      <c r="F25" s="63" t="s">
         <v>199</v>
       </c>
-      <c r="G25" s="73" t="s">
+      <c r="G25" s="63" t="s">
         <v>95</v>
       </c>
-      <c r="H25" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="I25" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="J25" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="K25" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="L25" s="73">
+      <c r="H25" s="63" t="s">
+        <v>198</v>
+      </c>
+      <c r="I25" s="63" t="s">
+        <v>198</v>
+      </c>
+      <c r="J25" s="63" t="s">
+        <v>198</v>
+      </c>
+      <c r="K25" s="63" t="s">
+        <v>198</v>
+      </c>
+      <c r="L25" s="63">
         <v>1</v>
       </c>
-      <c r="M25" s="73">
+      <c r="M25" s="63">
         <f t="shared" ref="M25" si="14">L25*5</f>
         <v>5</v>
       </c>
-      <c r="N25" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="O25" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="P25" s="74" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q25" s="74" t="s">
-        <v>198</v>
-      </c>
-      <c r="R25" s="73"/>
-      <c r="S25" s="75"/>
+      <c r="N25" s="63" t="s">
+        <v>198</v>
+      </c>
+      <c r="O25" s="63" t="s">
+        <v>198</v>
+      </c>
+      <c r="P25" s="64" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q25" s="64" t="s">
+        <v>198</v>
+      </c>
+      <c r="R25" s="63"/>
+      <c r="S25" s="65"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
@@ -3041,7 +3044,7 @@
       <c r="N26" s="37">
         <v>11</v>
       </c>
-      <c r="O26" s="70" t="s">
+      <c r="O26" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P26" s="38">
@@ -3097,7 +3100,7 @@
       <c r="N27" s="51">
         <v>10</v>
       </c>
-      <c r="O27" s="72" t="s">
+      <c r="O27" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P27" s="52">
@@ -3153,7 +3156,7 @@
       <c r="N28" s="37">
         <v>100</v>
       </c>
-      <c r="O28" s="70" t="s">
+      <c r="O28" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P28" s="38">
@@ -3184,7 +3187,7 @@
       <c r="F29" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="G29" s="71" t="s">
+      <c r="G29" s="61" t="s">
         <v>121</v>
       </c>
       <c r="H29" s="51" t="s">
@@ -3209,7 +3212,7 @@
       <c r="N29" s="51">
         <v>100</v>
       </c>
-      <c r="O29" s="72" t="s">
+      <c r="O29" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P29" s="52">
@@ -3265,7 +3268,7 @@
       <c r="N30" s="37">
         <v>100</v>
       </c>
-      <c r="O30" s="70" t="s">
+      <c r="O30" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P30" s="38">
@@ -3321,7 +3324,7 @@
       <c r="N31" s="51">
         <v>10</v>
       </c>
-      <c r="O31" s="72" t="s">
+      <c r="O31" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P31" s="52">
@@ -3377,7 +3380,7 @@
       <c r="N32" s="37">
         <v>100</v>
       </c>
-      <c r="O32" s="70" t="s">
+      <c r="O32" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P32" s="38">
@@ -3433,7 +3436,7 @@
       <c r="N33" s="51">
         <v>100</v>
       </c>
-      <c r="O33" s="72" t="s">
+      <c r="O33" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P33" s="52">
@@ -3489,7 +3492,7 @@
       <c r="N34" s="37">
         <v>100</v>
       </c>
-      <c r="O34" s="70" t="s">
+      <c r="O34" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P34" s="38">
@@ -3545,7 +3548,7 @@
       <c r="N35" s="51">
         <v>100</v>
       </c>
-      <c r="O35" s="72" t="s">
+      <c r="O35" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P35" s="52">
@@ -3576,7 +3579,7 @@
       <c r="F36" s="37" t="s">
         <v>101</v>
       </c>
-      <c r="G36" s="79" t="s">
+      <c r="G36" s="69" t="s">
         <v>128</v>
       </c>
       <c r="H36" s="37" t="s">
@@ -3601,7 +3604,7 @@
       <c r="N36" s="37">
         <v>100</v>
       </c>
-      <c r="O36" s="70" t="s">
+      <c r="O36" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P36" s="38">
@@ -3657,7 +3660,7 @@
       <c r="N37" s="51">
         <v>100</v>
       </c>
-      <c r="O37" s="72" t="s">
+      <c r="O37" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P37" s="52">
@@ -3679,53 +3682,53 @@
       <c r="C38" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="D38" s="76" t="s">
+      <c r="D38" s="66" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="76" t="s">
+      <c r="E38" s="66" t="s">
         <v>79</v>
       </c>
-      <c r="F38" s="76" t="s">
+      <c r="F38" s="66" t="s">
         <v>199</v>
       </c>
-      <c r="G38" s="76" t="s">
+      <c r="G38" s="66" t="s">
         <v>103</v>
       </c>
-      <c r="H38" s="76" t="s">
-        <v>198</v>
-      </c>
-      <c r="I38" s="76" t="s">
-        <v>198</v>
-      </c>
-      <c r="J38" s="76" t="s">
-        <v>198</v>
-      </c>
-      <c r="K38" s="76" t="s">
-        <v>198</v>
-      </c>
-      <c r="L38" s="76">
+      <c r="H38" s="66" t="s">
+        <v>198</v>
+      </c>
+      <c r="I38" s="66" t="s">
+        <v>198</v>
+      </c>
+      <c r="J38" s="66" t="s">
+        <v>198</v>
+      </c>
+      <c r="K38" s="66" t="s">
+        <v>198</v>
+      </c>
+      <c r="L38" s="66">
         <v>7</v>
       </c>
-      <c r="M38" s="76">
+      <c r="M38" s="66">
         <f>L38*5</f>
         <v>35</v>
       </c>
-      <c r="N38" s="76" t="s">
-        <v>198</v>
-      </c>
-      <c r="O38" s="76" t="s">
-        <v>198</v>
-      </c>
-      <c r="P38" s="77" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q38" s="77" t="s">
-        <v>198</v>
-      </c>
-      <c r="R38" s="76"/>
-      <c r="S38" s="75"/>
-    </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="N38" s="66" t="s">
+        <v>198</v>
+      </c>
+      <c r="O38" s="66" t="s">
+        <v>198</v>
+      </c>
+      <c r="P38" s="67" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q38" s="67" t="s">
+        <v>198</v>
+      </c>
+      <c r="R38" s="66"/>
+      <c r="S38" s="65"/>
+    </row>
+    <row r="39" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="47">
         <f t="shared" si="0"/>
@@ -3765,12 +3768,18 @@
         <f t="shared" ref="M39" si="27">L39*5</f>
         <v>5</v>
       </c>
-      <c r="N39" s="51"/>
-      <c r="O39" s="51"/>
-      <c r="P39" s="52"/>
+      <c r="N39" s="51">
+        <v>6</v>
+      </c>
+      <c r="O39" s="62" t="s">
+        <v>231</v>
+      </c>
+      <c r="P39" s="52">
+        <v>3.26</v>
+      </c>
       <c r="Q39" s="52">
         <f t="shared" ref="Q39" si="28">P39*N39</f>
-        <v>0</v>
+        <v>19.559999999999999</v>
       </c>
       <c r="R39" s="51"/>
       <c r="S39" s="59"/>
@@ -3818,7 +3827,7 @@
       <c r="N40" s="37">
         <v>6</v>
       </c>
-      <c r="O40" s="70" t="s">
+      <c r="O40" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P40" s="38">
@@ -3873,7 +3882,7 @@
       <c r="N41" s="37">
         <v>5</v>
       </c>
-      <c r="O41" s="70" t="s">
+      <c r="O41" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P41" s="38">
@@ -3928,7 +3937,7 @@
       <c r="N42" s="37">
         <v>5</v>
       </c>
-      <c r="O42" s="70" t="s">
+      <c r="O42" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P42" s="38">
@@ -3983,7 +3992,7 @@
       <c r="N43" s="37">
         <v>5</v>
       </c>
-      <c r="O43" s="70" t="s">
+      <c r="O43" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P43" s="38">
@@ -4038,7 +4047,7 @@
       <c r="N44" s="37">
         <v>5</v>
       </c>
-      <c r="O44" s="70" t="s">
+      <c r="O44" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P44" s="38">
@@ -4065,17 +4074,17 @@
       <c r="K45" s="45"/>
       <c r="L45" s="45"/>
       <c r="M45" s="45"/>
-      <c r="N45" s="68" t="s">
+      <c r="N45" s="84" t="s">
         <v>5</v>
       </c>
-      <c r="O45" s="69"/>
-      <c r="P45" s="69"/>
+      <c r="O45" s="85"/>
+      <c r="P45" s="85"/>
       <c r="Q45" s="48">
         <f>SUM(Q10:Q44)</f>
-        <v>29.805900000000001</v>
-      </c>
-      <c r="R45" s="64"/>
-      <c r="S45" s="65"/>
+        <v>49.365900000000003</v>
+      </c>
+      <c r="R45" s="80"/>
+      <c r="S45" s="81"/>
     </row>
     <row r="46" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
@@ -4091,17 +4100,17 @@
       <c r="K46" s="10"/>
       <c r="L46" s="10"/>
       <c r="M46" s="10"/>
-      <c r="N46" s="68" t="s">
+      <c r="N46" s="84" t="s">
         <v>6</v>
       </c>
-      <c r="O46" s="69"/>
-      <c r="P46" s="69"/>
+      <c r="O46" s="85"/>
+      <c r="P46" s="85"/>
       <c r="Q46" s="49">
         <f>Q45/5</f>
-        <v>5.9611800000000006</v>
-      </c>
-      <c r="R46" s="66"/>
-      <c r="S46" s="67"/>
+        <v>9.8731800000000014</v>
+      </c>
+      <c r="R46" s="82"/>
+      <c r="S46" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -4143,10 +4152,11 @@
     <hyperlink ref="O42" r:id="rId29"/>
     <hyperlink ref="O43" r:id="rId30"/>
     <hyperlink ref="O44" r:id="rId31"/>
+    <hyperlink ref="O39" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId32"/>
-  <drawing r:id="rId33"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId33"/>
+  <drawing r:id="rId34"/>
 </worksheet>
 </file>
 
@@ -4168,7 +4178,7 @@
     <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.5703125" customWidth="1"/>
     <col min="16" max="16" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="12.42578125" customWidth="1"/>
@@ -4186,15 +4196,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="61"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="76"/>
+      <c r="M1" s="76"/>
+      <c r="N1" s="76"/>
+      <c r="O1" s="76"/>
+      <c r="P1" s="76"/>
+      <c r="Q1" s="76"/>
+      <c r="R1" s="76"/>
+      <c r="S1" s="77"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -4244,7 +4254,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="62"/>
+      <c r="S3" s="78"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -4269,7 +4279,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="63"/>
+      <c r="S4" s="79"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -4294,7 +4304,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="63"/>
+      <c r="S5" s="79"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -4315,7 +4325,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="63"/>
+      <c r="S6" s="79"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -4336,7 +4346,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="63"/>
+      <c r="S7" s="79"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -4357,7 +4367,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="63"/>
+      <c r="S8" s="79"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -4416,8 +4426,8 @@
         <v>197</v>
       </c>
     </row>
-    <row r="10" spans="1:19" s="82" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="80"/>
+    <row r="10" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="70"/>
       <c r="B10" s="46">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
@@ -4459,7 +4469,7 @@
       <c r="N10" s="37">
         <v>20</v>
       </c>
-      <c r="O10" s="70" t="s">
+      <c r="O10" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P10" s="38">
@@ -4470,10 +4480,10 @@
         <v>0.74399999999999999</v>
       </c>
       <c r="R10" s="37"/>
-      <c r="S10" s="81"/>
-    </row>
-    <row r="11" spans="1:19" s="82" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="80"/>
+      <c r="S10" s="71"/>
+    </row>
+    <row r="11" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="70"/>
       <c r="B11" s="47">
         <f t="shared" ref="B11:B39" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
@@ -4490,7 +4500,7 @@
       <c r="F11" s="51" t="s">
         <v>83</v>
       </c>
-      <c r="G11" s="71" t="s">
+      <c r="G11" s="61" t="s">
         <v>108</v>
       </c>
       <c r="H11" s="51" t="s">
@@ -4509,13 +4519,13 @@
         <v>1</v>
       </c>
       <c r="M11" s="37">
-        <f t="shared" ref="M11:M44" si="1">L11*10</f>
+        <f t="shared" ref="M11:M40" si="1">L11*10</f>
         <v>10</v>
       </c>
       <c r="N11" s="51">
         <v>50</v>
       </c>
-      <c r="O11" s="72" t="s">
+      <c r="O11" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P11" s="52">
@@ -4528,8 +4538,8 @@
       <c r="R11" s="51"/>
       <c r="S11" s="51"/>
     </row>
-    <row r="12" spans="1:19" s="82" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="80"/>
+    <row r="12" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="70"/>
       <c r="B12" s="46">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
@@ -4571,7 +4581,7 @@
       <c r="N12" s="37">
         <v>100</v>
       </c>
-      <c r="O12" s="70" t="s">
+      <c r="O12" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P12" s="38">
@@ -4584,8 +4594,8 @@
       <c r="R12" s="37"/>
       <c r="S12" s="59"/>
     </row>
-    <row r="13" spans="1:19" s="82" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="80"/>
+    <row r="13" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="70"/>
       <c r="B13" s="47">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -4627,7 +4637,7 @@
       <c r="N13" s="51">
         <v>20</v>
       </c>
-      <c r="O13" s="72" t="s">
+      <c r="O13" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P13" s="52">
@@ -4640,8 +4650,8 @@
       <c r="R13" s="51"/>
       <c r="S13" s="59"/>
     </row>
-    <row r="14" spans="1:19" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A14" s="80"/>
+    <row r="14" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A14" s="70"/>
       <c r="B14" s="46">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
@@ -4683,7 +4693,7 @@
       <c r="N14" s="37">
         <v>50</v>
       </c>
-      <c r="O14" s="70" t="s">
+      <c r="O14" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P14" s="38">
@@ -4696,8 +4706,8 @@
       <c r="R14" s="37"/>
       <c r="S14" s="59"/>
     </row>
-    <row r="15" spans="1:19" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A15" s="80"/>
+    <row r="15" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A15" s="70"/>
       <c r="B15" s="47">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -4739,7 +4749,7 @@
       <c r="N15" s="51">
         <v>20</v>
       </c>
-      <c r="O15" s="72" t="s">
+      <c r="O15" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P15" s="52">
@@ -4752,8 +4762,8 @@
       <c r="R15" s="51"/>
       <c r="S15" s="59"/>
     </row>
-    <row r="16" spans="1:19" s="82" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="80"/>
+    <row r="16" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="70"/>
       <c r="B16" s="46">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
@@ -4795,7 +4805,7 @@
       <c r="N16" s="37">
         <v>100</v>
       </c>
-      <c r="O16" s="70" t="s">
+      <c r="O16" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P16" s="38">
@@ -4808,8 +4818,8 @@
       <c r="R16" s="37"/>
       <c r="S16" s="59"/>
     </row>
-    <row r="17" spans="1:19" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A17" s="80"/>
+    <row r="17" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A17" s="70"/>
       <c r="B17" s="47">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -4851,7 +4861,7 @@
       <c r="N17" s="51">
         <v>50</v>
       </c>
-      <c r="O17" s="72" t="s">
+      <c r="O17" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P17" s="52">
@@ -4864,8 +4874,8 @@
       <c r="R17" s="51"/>
       <c r="S17" s="59"/>
     </row>
-    <row r="18" spans="1:19" s="82" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A18" s="80"/>
+    <row r="18" spans="1:19" s="72" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A18" s="70"/>
       <c r="B18" s="46">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
@@ -4907,7 +4917,7 @@
       <c r="N18" s="37">
         <v>40</v>
       </c>
-      <c r="O18" s="70" t="s">
+      <c r="O18" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P18" s="38">
@@ -4920,8 +4930,8 @@
       <c r="R18" s="37"/>
       <c r="S18" s="59"/>
     </row>
-    <row r="19" spans="1:19" s="82" customFormat="1" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A19" s="80"/>
+    <row r="19" spans="1:19" s="72" customFormat="1" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A19" s="70"/>
       <c r="B19" s="47">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -4963,7 +4973,7 @@
       <c r="N19" s="51">
         <v>15</v>
       </c>
-      <c r="O19" s="72" t="s">
+      <c r="O19" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P19" s="52">
@@ -4976,8 +4986,8 @@
       <c r="R19" s="51"/>
       <c r="S19" s="59"/>
     </row>
-    <row r="20" spans="1:19" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A20" s="80"/>
+    <row r="20" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A20" s="70"/>
       <c r="B20" s="46">
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
@@ -5019,7 +5029,7 @@
       <c r="N20" s="37">
         <v>50</v>
       </c>
-      <c r="O20" s="70" t="s">
+      <c r="O20" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P20" s="38">
@@ -5032,8 +5042,8 @@
       <c r="R20" s="37"/>
       <c r="S20" s="59"/>
     </row>
-    <row r="21" spans="1:19" s="82" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="80"/>
+    <row r="21" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="70"/>
       <c r="B21" s="47">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -5075,7 +5085,7 @@
       <c r="N21" s="51">
         <v>15</v>
       </c>
-      <c r="O21" s="72" t="s">
+      <c r="O21" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P21" s="52">
@@ -5088,8 +5098,8 @@
       <c r="R21" s="51"/>
       <c r="S21" s="59"/>
     </row>
-    <row r="22" spans="1:19" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A22" s="80"/>
+    <row r="22" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A22" s="70"/>
       <c r="B22" s="46">
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
@@ -5131,7 +5141,7 @@
       <c r="N22" s="37">
         <v>15</v>
       </c>
-      <c r="O22" s="70" t="s">
+      <c r="O22" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P22" s="38">
@@ -5144,8 +5154,8 @@
       <c r="R22" s="37"/>
       <c r="S22" s="59"/>
     </row>
-    <row r="23" spans="1:19" s="82" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="80"/>
+    <row r="23" spans="1:19" s="72" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A23" s="70"/>
       <c r="B23" s="47">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -5153,54 +5163,54 @@
       <c r="C23" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="D23" s="71" t="s">
+      <c r="D23" s="61" t="s">
         <v>33</v>
       </c>
-      <c r="E23" s="71" t="s">
+      <c r="E23" s="61" t="s">
         <v>65</v>
       </c>
-      <c r="F23" s="71" t="s">
+      <c r="F23" s="61" t="s">
         <v>199</v>
       </c>
-      <c r="G23" s="71" t="s">
+      <c r="G23" s="61" t="s">
         <v>93</v>
       </c>
-      <c r="H23" s="71" t="s">
-        <v>198</v>
-      </c>
-      <c r="I23" s="71"/>
-      <c r="J23" s="71" t="s">
-        <v>198</v>
-      </c>
-      <c r="K23" s="71" t="s">
-        <v>198</v>
-      </c>
-      <c r="L23" s="71">
+      <c r="H23" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="I23" s="61"/>
+      <c r="J23" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="K23" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="L23" s="61">
         <v>6</v>
       </c>
-      <c r="M23" s="79">
+      <c r="M23" s="69">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
-      <c r="N23" s="71" t="s">
-        <v>198</v>
-      </c>
-      <c r="O23" s="71" t="s">
-        <v>198</v>
-      </c>
-      <c r="P23" s="83" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q23" s="83" t="s">
-        <v>198</v>
-      </c>
-      <c r="R23" s="84" t="s">
+      <c r="N23" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="O23" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="P23" s="73" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q23" s="73" t="s">
+        <v>198</v>
+      </c>
+      <c r="R23" s="74" t="s">
         <v>214</v>
       </c>
-      <c r="S23" s="75"/>
-    </row>
-    <row r="24" spans="1:19" s="82" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="80"/>
+      <c r="S23" s="65"/>
+    </row>
+    <row r="24" spans="1:19" s="72" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="70"/>
       <c r="B24" s="46">
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
@@ -5217,7 +5227,7 @@
       <c r="F24" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="G24" s="79" t="s">
+      <c r="G24" s="69" t="s">
         <v>117</v>
       </c>
       <c r="H24" s="37" t="s">
@@ -5242,7 +5252,7 @@
       <c r="N24" s="37">
         <v>100</v>
       </c>
-      <c r="O24" s="70" t="s">
+      <c r="O24" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P24" s="38">
@@ -5255,8 +5265,8 @@
       <c r="R24" s="37"/>
       <c r="S24" s="59"/>
     </row>
-    <row r="25" spans="1:19" s="82" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A25" s="80"/>
+    <row r="25" spans="1:19" s="72" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="70"/>
       <c r="B25" s="47">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -5264,56 +5274,56 @@
       <c r="C25" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="D25" s="71" t="s">
+      <c r="D25" s="61" t="s">
         <v>35</v>
       </c>
-      <c r="E25" s="71" t="s">
+      <c r="E25" s="61" t="s">
         <v>65</v>
       </c>
-      <c r="F25" s="71" t="s">
+      <c r="F25" s="61" t="s">
         <v>199</v>
       </c>
-      <c r="G25" s="71" t="s">
+      <c r="G25" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="H25" s="71" t="s">
-        <v>198</v>
-      </c>
-      <c r="I25" s="71" t="s">
-        <v>198</v>
-      </c>
-      <c r="J25" s="71" t="s">
-        <v>198</v>
-      </c>
-      <c r="K25" s="71" t="s">
-        <v>198</v>
-      </c>
-      <c r="L25" s="71">
+      <c r="H25" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="I25" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="J25" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="K25" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="L25" s="61">
         <v>1</v>
       </c>
-      <c r="M25" s="78">
+      <c r="M25" s="68">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N25" s="71" t="s">
-        <v>198</v>
-      </c>
-      <c r="O25" s="71" t="s">
-        <v>198</v>
-      </c>
-      <c r="P25" s="83" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q25" s="83" t="s">
-        <v>198</v>
-      </c>
-      <c r="R25" s="84" t="s">
+      <c r="N25" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="O25" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="P25" s="73" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q25" s="73" t="s">
+        <v>198</v>
+      </c>
+      <c r="R25" s="74" t="s">
         <v>214</v>
       </c>
-      <c r="S25" s="75"/>
-    </row>
-    <row r="26" spans="1:19" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A26" s="80"/>
+      <c r="S25" s="65"/>
+    </row>
+    <row r="26" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A26" s="70"/>
       <c r="B26" s="46">
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
@@ -5330,7 +5340,7 @@
       <c r="F26" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="G26" s="79" t="s">
+      <c r="G26" s="69" t="s">
         <v>118</v>
       </c>
       <c r="H26" s="37" t="s">
@@ -5355,7 +5365,7 @@
       <c r="N26" s="37">
         <v>21</v>
       </c>
-      <c r="O26" s="70" t="s">
+      <c r="O26" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P26" s="38">
@@ -5368,8 +5378,8 @@
       <c r="R26" s="37"/>
       <c r="S26" s="59"/>
     </row>
-    <row r="27" spans="1:19" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A27" s="80"/>
+    <row r="27" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A27" s="70"/>
       <c r="B27" s="47">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -5411,7 +5421,7 @@
       <c r="N27" s="51">
         <v>20</v>
       </c>
-      <c r="O27" s="72" t="s">
+      <c r="O27" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P27" s="52">
@@ -5424,8 +5434,8 @@
       <c r="R27" s="51"/>
       <c r="S27" s="59"/>
     </row>
-    <row r="28" spans="1:19" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A28" s="80"/>
+    <row r="28" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A28" s="70"/>
       <c r="B28" s="46">
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
@@ -5467,7 +5477,7 @@
       <c r="N28" s="37">
         <v>100</v>
       </c>
-      <c r="O28" s="70" t="s">
+      <c r="O28" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P28" s="38">
@@ -5480,8 +5490,8 @@
       <c r="R28" s="51"/>
       <c r="S28" s="59"/>
     </row>
-    <row r="29" spans="1:19" s="82" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="80"/>
+    <row r="29" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="70"/>
       <c r="B29" s="47">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -5498,7 +5508,7 @@
       <c r="F29" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="G29" s="71" t="s">
+      <c r="G29" s="61" t="s">
         <v>121</v>
       </c>
       <c r="H29" s="51" t="s">
@@ -5523,7 +5533,7 @@
       <c r="N29" s="51">
         <v>100</v>
       </c>
-      <c r="O29" s="72" t="s">
+      <c r="O29" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P29" s="52">
@@ -5536,8 +5546,8 @@
       <c r="R29" s="51"/>
       <c r="S29" s="59"/>
     </row>
-    <row r="30" spans="1:19" s="82" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="80"/>
+    <row r="30" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="70"/>
       <c r="B30" s="46">
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
@@ -5579,7 +5589,7 @@
       <c r="N30" s="37">
         <v>100</v>
       </c>
-      <c r="O30" s="70" t="s">
+      <c r="O30" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P30" s="38">
@@ -5592,8 +5602,8 @@
       <c r="R30" s="37"/>
       <c r="S30" s="59"/>
     </row>
-    <row r="31" spans="1:19" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A31" s="80"/>
+    <row r="31" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A31" s="70"/>
       <c r="B31" s="47">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -5635,7 +5645,7 @@
       <c r="N31" s="51">
         <v>15</v>
       </c>
-      <c r="O31" s="72" t="s">
+      <c r="O31" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P31" s="52">
@@ -5648,8 +5658,8 @@
       <c r="R31" s="51"/>
       <c r="S31" s="59"/>
     </row>
-    <row r="32" spans="1:19" s="82" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="80"/>
+    <row r="32" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="70"/>
       <c r="B32" s="46">
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
@@ -5691,7 +5701,7 @@
       <c r="N32" s="37">
         <v>100</v>
       </c>
-      <c r="O32" s="70" t="s">
+      <c r="O32" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P32" s="38">
@@ -5704,8 +5714,8 @@
       <c r="R32" s="37"/>
       <c r="S32" s="59"/>
     </row>
-    <row r="33" spans="1:19" s="82" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="80"/>
+    <row r="33" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="70"/>
       <c r="B33" s="47">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -5747,7 +5757,7 @@
       <c r="N33" s="51">
         <v>100</v>
       </c>
-      <c r="O33" s="72" t="s">
+      <c r="O33" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P33" s="52">
@@ -5760,8 +5770,8 @@
       <c r="R33" s="51"/>
       <c r="S33" s="59"/>
     </row>
-    <row r="34" spans="1:19" s="82" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="80"/>
+    <row r="34" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="70"/>
       <c r="B34" s="46">
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
@@ -5803,7 +5813,7 @@
       <c r="N34" s="37">
         <v>100</v>
       </c>
-      <c r="O34" s="70" t="s">
+      <c r="O34" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P34" s="38">
@@ -5816,8 +5826,8 @@
       <c r="R34" s="37"/>
       <c r="S34" s="59"/>
     </row>
-    <row r="35" spans="1:19" s="82" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="80"/>
+    <row r="35" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="70"/>
       <c r="B35" s="47">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -5859,7 +5869,7 @@
       <c r="N35" s="51">
         <v>100</v>
       </c>
-      <c r="O35" s="72" t="s">
+      <c r="O35" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P35" s="52">
@@ -5872,8 +5882,8 @@
       <c r="R35" s="51"/>
       <c r="S35" s="59"/>
     </row>
-    <row r="36" spans="1:19" s="82" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="80"/>
+    <row r="36" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="70"/>
       <c r="B36" s="46">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
@@ -5890,7 +5900,7 @@
       <c r="F36" s="37" t="s">
         <v>101</v>
       </c>
-      <c r="G36" s="79" t="s">
+      <c r="G36" s="69" t="s">
         <v>128</v>
       </c>
       <c r="H36" s="37" t="s">
@@ -5915,7 +5925,7 @@
       <c r="N36" s="37">
         <v>100</v>
       </c>
-      <c r="O36" s="70" t="s">
+      <c r="O36" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P36" s="38">
@@ -5928,8 +5938,8 @@
       <c r="R36" s="37"/>
       <c r="S36" s="59"/>
     </row>
-    <row r="37" spans="1:19" s="82" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="80"/>
+    <row r="37" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="70"/>
       <c r="B37" s="47">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -5971,7 +5981,7 @@
       <c r="N37" s="51">
         <v>100</v>
       </c>
-      <c r="O37" s="72" t="s">
+      <c r="O37" s="62" t="s">
         <v>200</v>
       </c>
       <c r="P37" s="52">
@@ -5984,8 +5994,8 @@
       <c r="R37" s="51"/>
       <c r="S37" s="59"/>
     </row>
-    <row r="38" spans="1:19" s="82" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A38" s="80"/>
+    <row r="38" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="70"/>
       <c r="B38" s="46">
         <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
@@ -5993,56 +6003,56 @@
       <c r="C38" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="D38" s="79" t="s">
+      <c r="D38" s="69" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="79" t="s">
+      <c r="E38" s="69" t="s">
         <v>79</v>
       </c>
-      <c r="F38" s="79" t="s">
+      <c r="F38" s="69" t="s">
         <v>199</v>
       </c>
-      <c r="G38" s="79" t="s">
+      <c r="G38" s="69" t="s">
         <v>103</v>
       </c>
-      <c r="H38" s="79" t="s">
-        <v>198</v>
-      </c>
-      <c r="I38" s="79" t="s">
-        <v>198</v>
-      </c>
-      <c r="J38" s="79" t="s">
-        <v>198</v>
-      </c>
-      <c r="K38" s="79" t="s">
-        <v>198</v>
-      </c>
-      <c r="L38" s="79">
+      <c r="H38" s="69" t="s">
+        <v>198</v>
+      </c>
+      <c r="I38" s="69" t="s">
+        <v>198</v>
+      </c>
+      <c r="J38" s="69" t="s">
+        <v>198</v>
+      </c>
+      <c r="K38" s="69" t="s">
+        <v>198</v>
+      </c>
+      <c r="L38" s="69">
         <v>7</v>
       </c>
-      <c r="M38" s="79">
+      <c r="M38" s="69">
         <f t="shared" si="1"/>
         <v>70</v>
       </c>
-      <c r="N38" s="79" t="s">
-        <v>198</v>
-      </c>
-      <c r="O38" s="79" t="s">
-        <v>198</v>
-      </c>
-      <c r="P38" s="85" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q38" s="85" t="s">
-        <v>198</v>
-      </c>
-      <c r="R38" s="84" t="s">
+      <c r="N38" s="69" t="s">
+        <v>198</v>
+      </c>
+      <c r="O38" s="69" t="s">
+        <v>198</v>
+      </c>
+      <c r="P38" s="75" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q38" s="75" t="s">
+        <v>198</v>
+      </c>
+      <c r="R38" s="74" t="s">
         <v>214</v>
       </c>
-      <c r="S38" s="75"/>
-    </row>
-    <row r="39" spans="1:19" s="82" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A39" s="80"/>
+      <c r="S38" s="65"/>
+    </row>
+    <row r="39" spans="1:19" s="72" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A39" s="70"/>
       <c r="B39" s="47">
         <f t="shared" si="0"/>
         <v>30</v>
@@ -6081,18 +6091,24 @@
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N39" s="51"/>
-      <c r="O39" s="51"/>
-      <c r="P39" s="52"/>
+      <c r="N39" s="51">
+        <v>11</v>
+      </c>
+      <c r="O39" s="62" t="s">
+        <v>231</v>
+      </c>
+      <c r="P39" s="52">
+        <v>2.93</v>
+      </c>
       <c r="Q39" s="52">
         <f t="shared" ref="Q39" si="14">P39*N39</f>
-        <v>0</v>
+        <v>32.230000000000004</v>
       </c>
       <c r="R39" s="51"/>
       <c r="S39" s="59"/>
     </row>
-    <row r="40" spans="1:19" s="82" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="80"/>
+    <row r="40" spans="1:19" s="72" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="70"/>
       <c r="B40" s="46">
         <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
@@ -6134,7 +6150,7 @@
       <c r="N40" s="37">
         <v>11</v>
       </c>
-      <c r="O40" s="70" t="s">
+      <c r="O40" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P40" s="38">
@@ -6189,7 +6205,7 @@
       <c r="N41" s="37">
         <v>5</v>
       </c>
-      <c r="O41" s="70" t="s">
+      <c r="O41" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P41" s="38">
@@ -6244,7 +6260,7 @@
       <c r="N42" s="37">
         <v>5</v>
       </c>
-      <c r="O42" s="70" t="s">
+      <c r="O42" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P42" s="38">
@@ -6299,7 +6315,7 @@
       <c r="N43" s="37">
         <v>5</v>
       </c>
-      <c r="O43" s="70" t="s">
+      <c r="O43" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P43" s="38">
@@ -6354,7 +6370,7 @@
       <c r="N44" s="37">
         <v>5</v>
       </c>
-      <c r="O44" s="70" t="s">
+      <c r="O44" s="60" t="s">
         <v>200</v>
       </c>
       <c r="P44" s="38">
@@ -6381,17 +6397,17 @@
       <c r="K45" s="45"/>
       <c r="L45" s="45"/>
       <c r="M45" s="45"/>
-      <c r="N45" s="68" t="s">
+      <c r="N45" s="84" t="s">
         <v>5</v>
       </c>
-      <c r="O45" s="69"/>
-      <c r="P45" s="69"/>
+      <c r="O45" s="85"/>
+      <c r="P45" s="85"/>
       <c r="Q45" s="48">
         <f>SUM(Q10:Q44)</f>
-        <v>46.061200000000007</v>
-      </c>
-      <c r="R45" s="64"/>
-      <c r="S45" s="65"/>
+        <v>78.291200000000003</v>
+      </c>
+      <c r="R45" s="80"/>
+      <c r="S45" s="81"/>
     </row>
     <row r="46" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
@@ -6407,17 +6423,17 @@
       <c r="K46" s="10"/>
       <c r="L46" s="10"/>
       <c r="M46" s="10"/>
-      <c r="N46" s="68" t="s">
+      <c r="N46" s="84" t="s">
         <v>6</v>
       </c>
-      <c r="O46" s="69"/>
-      <c r="P46" s="69"/>
+      <c r="O46" s="85"/>
+      <c r="P46" s="85"/>
       <c r="Q46" s="49">
         <f>Q45/10</f>
-        <v>4.6061200000000007</v>
-      </c>
-      <c r="R46" s="66"/>
-      <c r="S46" s="67"/>
+        <v>7.8291200000000005</v>
+      </c>
+      <c r="R46" s="82"/>
+      <c r="S46" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -6459,8 +6475,9 @@
     <hyperlink ref="O42" r:id="rId29"/>
     <hyperlink ref="O43" r:id="rId30"/>
     <hyperlink ref="O44" r:id="rId31"/>
+    <hyperlink ref="O39" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId32"/>
+  <drawing r:id="rId33"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#5 100 Boards eSaprk BOM Added.
</commit_message>
<xml_diff>
--- a/Design Files/BOM/eSpark-BOM-BMS-v1.0.xlsx
+++ b/Design Files/BOM/eSpark-BOM-BMS-v1.0.xlsx
@@ -9,18 +9,19 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
     <sheet name="10 Boards" sheetId="2" r:id="rId2"/>
+    <sheet name="100 Boards" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1163" uniqueCount="236">
   <si>
     <t>Component list</t>
   </si>
@@ -715,7 +716,19 @@
     <t>C394024</t>
   </si>
   <si>
-    <t>Custom Supplier</t>
+    <t>Quantity (100 Boards)</t>
+  </si>
+  <si>
+    <t>MOQ (100 Boards)</t>
+  </si>
+  <si>
+    <t>Unit Cost (100 Boards)</t>
+  </si>
+  <si>
+    <t>Total Cost (100 Boards)</t>
+  </si>
+  <si>
+    <t>Chipsmall</t>
   </si>
 </sst>
 </file>
@@ -727,7 +740,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -883,13 +896,6 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <strike/>
-      <sz val="9"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1210,7 +1216,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1374,31 +1380,28 @@
     <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="25" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="24" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="25" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="24" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1410,13 +1413,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="24" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="23" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="24" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="23" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1450,6 +1453,29 @@
     <xf numFmtId="0" fontId="20" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1571,6 +1597,60 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="20897850" y="620017"/>
+          <a:ext cx="1714500" cy="1104008"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>10417</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>1724025</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19088100" y="620017"/>
           <a:ext cx="1714500" cy="1104008"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1881,15 +1961,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="76"/>
-      <c r="L1" s="76"/>
-      <c r="M1" s="76"/>
-      <c r="N1" s="76"/>
-      <c r="O1" s="76"/>
-      <c r="P1" s="76"/>
-      <c r="Q1" s="76"/>
-      <c r="R1" s="76"/>
-      <c r="S1" s="77"/>
+      <c r="K1" s="75"/>
+      <c r="L1" s="75"/>
+      <c r="M1" s="75"/>
+      <c r="N1" s="75"/>
+      <c r="O1" s="75"/>
+      <c r="P1" s="75"/>
+      <c r="Q1" s="75"/>
+      <c r="R1" s="75"/>
+      <c r="S1" s="76"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1939,7 +2019,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="78"/>
+      <c r="S3" s="77"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1964,7 +2044,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="79"/>
+      <c r="S4" s="78"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1989,7 +2069,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="79"/>
+      <c r="S5" s="78"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2010,7 +2090,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="79"/>
+      <c r="S6" s="78"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2031,7 +2111,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="79"/>
+      <c r="S7" s="78"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2052,7 +2132,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="79"/>
+      <c r="S8" s="78"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2910,7 +2990,7 @@
       <c r="F24" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="G24" s="69" t="s">
+      <c r="G24" s="68" t="s">
         <v>117</v>
       </c>
       <c r="H24" s="37" t="s">
@@ -3579,7 +3659,7 @@
       <c r="F36" s="37" t="s">
         <v>101</v>
       </c>
-      <c r="G36" s="69" t="s">
+      <c r="G36" s="68" t="s">
         <v>128</v>
       </c>
       <c r="H36" s="37" t="s">
@@ -3728,7 +3808,7 @@
       <c r="R38" s="66"/>
       <c r="S38" s="65"/>
     </row>
-    <row r="39" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="B39" s="47">
         <f t="shared" si="0"/>
@@ -3772,14 +3852,14 @@
         <v>6</v>
       </c>
       <c r="O39" s="62" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="P39" s="52">
-        <v>3.26</v>
+        <v>2.0510000000000002</v>
       </c>
       <c r="Q39" s="52">
         <f t="shared" ref="Q39" si="28">P39*N39</f>
-        <v>19.559999999999999</v>
+        <v>12.306000000000001</v>
       </c>
       <c r="R39" s="51"/>
       <c r="S39" s="59"/>
@@ -4074,17 +4154,17 @@
       <c r="K45" s="45"/>
       <c r="L45" s="45"/>
       <c r="M45" s="45"/>
-      <c r="N45" s="84" t="s">
+      <c r="N45" s="83" t="s">
         <v>5</v>
       </c>
-      <c r="O45" s="85"/>
-      <c r="P45" s="85"/>
+      <c r="O45" s="84"/>
+      <c r="P45" s="84"/>
       <c r="Q45" s="48">
         <f>SUM(Q10:Q44)</f>
-        <v>49.365900000000003</v>
-      </c>
-      <c r="R45" s="80"/>
-      <c r="S45" s="81"/>
+        <v>42.111900000000006</v>
+      </c>
+      <c r="R45" s="79"/>
+      <c r="S45" s="80"/>
     </row>
     <row r="46" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
@@ -4100,17 +4180,17 @@
       <c r="K46" s="10"/>
       <c r="L46" s="10"/>
       <c r="M46" s="10"/>
-      <c r="N46" s="84" t="s">
+      <c r="N46" s="83" t="s">
         <v>6</v>
       </c>
-      <c r="O46" s="85"/>
-      <c r="P46" s="85"/>
+      <c r="O46" s="84"/>
+      <c r="P46" s="84"/>
       <c r="Q46" s="49">
         <f>Q45/5</f>
-        <v>9.8731800000000014</v>
-      </c>
-      <c r="R46" s="82"/>
-      <c r="S46" s="83"/>
+        <v>8.4223800000000004</v>
+      </c>
+      <c r="R46" s="81"/>
+      <c r="S46" s="82"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -4168,7 +4248,7 @@
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" customWidth="1"/>
     <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25" customWidth="1"/>
+    <col min="5" max="5" width="29.5703125" customWidth="1"/>
     <col min="6" max="6" width="13.140625" customWidth="1"/>
     <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -4196,15 +4276,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="76"/>
-      <c r="L1" s="76"/>
-      <c r="M1" s="76"/>
-      <c r="N1" s="76"/>
-      <c r="O1" s="76"/>
-      <c r="P1" s="76"/>
-      <c r="Q1" s="76"/>
-      <c r="R1" s="76"/>
-      <c r="S1" s="77"/>
+      <c r="K1" s="75"/>
+      <c r="L1" s="75"/>
+      <c r="M1" s="75"/>
+      <c r="N1" s="75"/>
+      <c r="O1" s="75"/>
+      <c r="P1" s="75"/>
+      <c r="Q1" s="75"/>
+      <c r="R1" s="75"/>
+      <c r="S1" s="76"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -4254,7 +4334,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="78"/>
+      <c r="S3" s="77"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -4279,7 +4359,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="79"/>
+      <c r="S4" s="78"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -4304,7 +4384,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="79"/>
+      <c r="S5" s="78"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -4325,7 +4405,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="79"/>
+      <c r="S6" s="78"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -4346,7 +4426,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="79"/>
+      <c r="S7" s="78"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -4367,7 +4447,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="79"/>
+      <c r="S8" s="78"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -4426,8 +4506,8 @@
         <v>197</v>
       </c>
     </row>
-    <row r="10" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="70"/>
+    <row r="10" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="69"/>
       <c r="B10" s="46">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
@@ -4480,10 +4560,10 @@
         <v>0.74399999999999999</v>
       </c>
       <c r="R10" s="37"/>
-      <c r="S10" s="71"/>
-    </row>
-    <row r="11" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="70"/>
+      <c r="S10" s="70"/>
+    </row>
+    <row r="11" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="69"/>
       <c r="B11" s="47">
         <f t="shared" ref="B11:B39" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
@@ -4538,8 +4618,8 @@
       <c r="R11" s="51"/>
       <c r="S11" s="51"/>
     </row>
-    <row r="12" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="70"/>
+    <row r="12" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="69"/>
       <c r="B12" s="46">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
@@ -4594,8 +4674,8 @@
       <c r="R12" s="37"/>
       <c r="S12" s="59"/>
     </row>
-    <row r="13" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="70"/>
+    <row r="13" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="69"/>
       <c r="B13" s="47">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -4650,8 +4730,8 @@
       <c r="R13" s="51"/>
       <c r="S13" s="59"/>
     </row>
-    <row r="14" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A14" s="70"/>
+    <row r="14" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A14" s="69"/>
       <c r="B14" s="46">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
@@ -4706,8 +4786,8 @@
       <c r="R14" s="37"/>
       <c r="S14" s="59"/>
     </row>
-    <row r="15" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A15" s="70"/>
+    <row r="15" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A15" s="69"/>
       <c r="B15" s="47">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -4762,8 +4842,8 @@
       <c r="R15" s="51"/>
       <c r="S15" s="59"/>
     </row>
-    <row r="16" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="70"/>
+    <row r="16" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="69"/>
       <c r="B16" s="46">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
@@ -4818,8 +4898,8 @@
       <c r="R16" s="37"/>
       <c r="S16" s="59"/>
     </row>
-    <row r="17" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A17" s="70"/>
+    <row r="17" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A17" s="69"/>
       <c r="B17" s="47">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -4874,8 +4954,8 @@
       <c r="R17" s="51"/>
       <c r="S17" s="59"/>
     </row>
-    <row r="18" spans="1:19" s="72" customFormat="1" ht="60" x14ac:dyDescent="0.25">
-      <c r="A18" s="70"/>
+    <row r="18" spans="1:19" s="71" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A18" s="69"/>
       <c r="B18" s="46">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
@@ -4930,8 +5010,8 @@
       <c r="R18" s="37"/>
       <c r="S18" s="59"/>
     </row>
-    <row r="19" spans="1:19" s="72" customFormat="1" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A19" s="70"/>
+    <row r="19" spans="1:19" s="71" customFormat="1" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A19" s="69"/>
       <c r="B19" s="47">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -4986,8 +5066,8 @@
       <c r="R19" s="51"/>
       <c r="S19" s="59"/>
     </row>
-    <row r="20" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A20" s="70"/>
+    <row r="20" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A20" s="69"/>
       <c r="B20" s="46">
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
@@ -5042,8 +5122,8 @@
       <c r="R20" s="37"/>
       <c r="S20" s="59"/>
     </row>
-    <row r="21" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="70"/>
+    <row r="21" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="69"/>
       <c r="B21" s="47">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -5098,8 +5178,8 @@
       <c r="R21" s="51"/>
       <c r="S21" s="59"/>
     </row>
-    <row r="22" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A22" s="70"/>
+    <row r="22" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A22" s="69"/>
       <c r="B22" s="46">
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
@@ -5154,8 +5234,8 @@
       <c r="R22" s="37"/>
       <c r="S22" s="59"/>
     </row>
-    <row r="23" spans="1:19" s="72" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="70"/>
+    <row r="23" spans="1:19" s="71" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A23" s="69"/>
       <c r="B23" s="47">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -5188,7 +5268,7 @@
       <c r="L23" s="61">
         <v>6</v>
       </c>
-      <c r="M23" s="69">
+      <c r="M23" s="68">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
@@ -5198,19 +5278,19 @@
       <c r="O23" s="61" t="s">
         <v>198</v>
       </c>
-      <c r="P23" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q23" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="R23" s="74" t="s">
+      <c r="P23" s="72" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q23" s="72" t="s">
+        <v>198</v>
+      </c>
+      <c r="R23" s="73" t="s">
         <v>214</v>
       </c>
       <c r="S23" s="65"/>
     </row>
-    <row r="24" spans="1:19" s="72" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="70"/>
+    <row r="24" spans="1:19" s="71" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="69"/>
       <c r="B24" s="46">
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
@@ -5227,7 +5307,7 @@
       <c r="F24" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="G24" s="69" t="s">
+      <c r="G24" s="68" t="s">
         <v>117</v>
       </c>
       <c r="H24" s="37" t="s">
@@ -5265,8 +5345,8 @@
       <c r="R24" s="37"/>
       <c r="S24" s="59"/>
     </row>
-    <row r="25" spans="1:19" s="72" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A25" s="70"/>
+    <row r="25" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="69"/>
       <c r="B25" s="47">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -5301,7 +5381,7 @@
       <c r="L25" s="61">
         <v>1</v>
       </c>
-      <c r="M25" s="68">
+      <c r="M25" s="61">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
@@ -5311,19 +5391,19 @@
       <c r="O25" s="61" t="s">
         <v>198</v>
       </c>
-      <c r="P25" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q25" s="73" t="s">
-        <v>198</v>
-      </c>
-      <c r="R25" s="74" t="s">
+      <c r="P25" s="72" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q25" s="72" t="s">
+        <v>198</v>
+      </c>
+      <c r="R25" s="73" t="s">
         <v>214</v>
       </c>
       <c r="S25" s="65"/>
     </row>
-    <row r="26" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A26" s="70"/>
+    <row r="26" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A26" s="69"/>
       <c r="B26" s="46">
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
@@ -5340,7 +5420,7 @@
       <c r="F26" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="G26" s="69" t="s">
+      <c r="G26" s="68" t="s">
         <v>118</v>
       </c>
       <c r="H26" s="37" t="s">
@@ -5378,8 +5458,8 @@
       <c r="R26" s="37"/>
       <c r="S26" s="59"/>
     </row>
-    <row r="27" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A27" s="70"/>
+    <row r="27" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A27" s="69"/>
       <c r="B27" s="47">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -5434,8 +5514,8 @@
       <c r="R27" s="51"/>
       <c r="S27" s="59"/>
     </row>
-    <row r="28" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A28" s="70"/>
+    <row r="28" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A28" s="69"/>
       <c r="B28" s="46">
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
@@ -5490,8 +5570,8 @@
       <c r="R28" s="51"/>
       <c r="S28" s="59"/>
     </row>
-    <row r="29" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="70"/>
+    <row r="29" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="69"/>
       <c r="B29" s="47">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -5546,8 +5626,8 @@
       <c r="R29" s="51"/>
       <c r="S29" s="59"/>
     </row>
-    <row r="30" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="70"/>
+    <row r="30" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="69"/>
       <c r="B30" s="46">
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
@@ -5602,8 +5682,8 @@
       <c r="R30" s="37"/>
       <c r="S30" s="59"/>
     </row>
-    <row r="31" spans="1:19" s="72" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A31" s="70"/>
+    <row r="31" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A31" s="69"/>
       <c r="B31" s="47">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -5658,8 +5738,8 @@
       <c r="R31" s="51"/>
       <c r="S31" s="59"/>
     </row>
-    <row r="32" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="70"/>
+    <row r="32" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="69"/>
       <c r="B32" s="46">
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
@@ -5714,8 +5794,8 @@
       <c r="R32" s="37"/>
       <c r="S32" s="59"/>
     </row>
-    <row r="33" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="70"/>
+    <row r="33" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="69"/>
       <c r="B33" s="47">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -5770,8 +5850,8 @@
       <c r="R33" s="51"/>
       <c r="S33" s="59"/>
     </row>
-    <row r="34" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="70"/>
+    <row r="34" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="69"/>
       <c r="B34" s="46">
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
@@ -5826,8 +5906,8 @@
       <c r="R34" s="37"/>
       <c r="S34" s="59"/>
     </row>
-    <row r="35" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="70"/>
+    <row r="35" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="69"/>
       <c r="B35" s="47">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -5882,8 +5962,8 @@
       <c r="R35" s="51"/>
       <c r="S35" s="59"/>
     </row>
-    <row r="36" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="70"/>
+    <row r="36" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="69"/>
       <c r="B36" s="46">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
@@ -5900,7 +5980,7 @@
       <c r="F36" s="37" t="s">
         <v>101</v>
       </c>
-      <c r="G36" s="69" t="s">
+      <c r="G36" s="68" t="s">
         <v>128</v>
       </c>
       <c r="H36" s="37" t="s">
@@ -5938,8 +6018,8 @@
       <c r="R36" s="37"/>
       <c r="S36" s="59"/>
     </row>
-    <row r="37" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="70"/>
+    <row r="37" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="69"/>
       <c r="B37" s="47">
         <f t="shared" si="0"/>
         <v>28</v>
@@ -5994,8 +6074,8 @@
       <c r="R37" s="51"/>
       <c r="S37" s="59"/>
     </row>
-    <row r="38" spans="1:19" s="72" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="70"/>
+    <row r="38" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="69"/>
       <c r="B38" s="46">
         <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
@@ -6003,112 +6083,112 @@
       <c r="C38" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="D38" s="69" t="s">
+      <c r="D38" s="68" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="69" t="s">
+      <c r="E38" s="68" t="s">
         <v>79</v>
       </c>
-      <c r="F38" s="69" t="s">
+      <c r="F38" s="68" t="s">
         <v>199</v>
       </c>
-      <c r="G38" s="69" t="s">
+      <c r="G38" s="68" t="s">
         <v>103</v>
       </c>
-      <c r="H38" s="69" t="s">
-        <v>198</v>
-      </c>
-      <c r="I38" s="69" t="s">
-        <v>198</v>
-      </c>
-      <c r="J38" s="69" t="s">
-        <v>198</v>
-      </c>
-      <c r="K38" s="69" t="s">
-        <v>198</v>
-      </c>
-      <c r="L38" s="69">
+      <c r="H38" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="I38" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="J38" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="K38" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="L38" s="68">
         <v>7</v>
       </c>
-      <c r="M38" s="69">
+      <c r="M38" s="68">
         <f t="shared" si="1"/>
         <v>70</v>
       </c>
-      <c r="N38" s="69" t="s">
-        <v>198</v>
-      </c>
-      <c r="O38" s="69" t="s">
-        <v>198</v>
-      </c>
-      <c r="P38" s="75" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q38" s="75" t="s">
-        <v>198</v>
-      </c>
-      <c r="R38" s="74" t="s">
+      <c r="N38" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="O38" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="P38" s="74" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q38" s="74" t="s">
+        <v>198</v>
+      </c>
+      <c r="R38" s="73" t="s">
         <v>214</v>
       </c>
       <c r="S38" s="65"/>
     </row>
-    <row r="39" spans="1:19" s="72" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A39" s="70"/>
-      <c r="B39" s="47">
+    <row r="39" spans="1:19" s="87" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="85"/>
+      <c r="B39" s="88">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C39" s="54" t="s">
+      <c r="C39" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="D39" s="51" t="s">
+      <c r="D39" s="89" t="s">
         <v>49</v>
       </c>
-      <c r="E39" s="51" t="s">
+      <c r="E39" s="89" t="s">
         <v>80</v>
       </c>
-      <c r="F39" s="51" t="s">
+      <c r="F39" s="89" t="s">
         <v>104</v>
       </c>
-      <c r="G39" s="51" t="s">
+      <c r="G39" s="89" t="s">
         <v>130</v>
       </c>
-      <c r="H39" s="51" t="s">
+      <c r="H39" s="89" t="s">
         <v>146</v>
       </c>
-      <c r="I39" s="51" t="s">
-        <v>198</v>
-      </c>
-      <c r="J39" s="51" t="s">
-        <v>198</v>
-      </c>
-      <c r="K39" s="51" t="s">
-        <v>198</v>
-      </c>
-      <c r="L39" s="51">
+      <c r="I39" s="89" t="s">
+        <v>198</v>
+      </c>
+      <c r="J39" s="89" t="s">
+        <v>198</v>
+      </c>
+      <c r="K39" s="89" t="s">
+        <v>198</v>
+      </c>
+      <c r="L39" s="89">
         <v>1</v>
       </c>
-      <c r="M39" s="37">
+      <c r="M39" s="86">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N39" s="51">
+      <c r="N39" s="89">
         <v>11</v>
       </c>
-      <c r="O39" s="62" t="s">
-        <v>231</v>
-      </c>
-      <c r="P39" s="52">
-        <v>2.93</v>
-      </c>
-      <c r="Q39" s="52">
+      <c r="O39" s="90" t="s">
+        <v>235</v>
+      </c>
+      <c r="P39" s="91">
+        <v>2.0510000000000002</v>
+      </c>
+      <c r="Q39" s="91">
         <f t="shared" ref="Q39" si="14">P39*N39</f>
-        <v>32.230000000000004</v>
-      </c>
-      <c r="R39" s="51"/>
-      <c r="S39" s="59"/>
-    </row>
-    <row r="40" spans="1:19" s="72" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="70"/>
+        <v>22.561</v>
+      </c>
+      <c r="R39" s="89"/>
+      <c r="S39" s="92"/>
+    </row>
+    <row r="40" spans="1:19" s="71" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="69"/>
       <c r="B40" s="46">
         <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
@@ -6397,17 +6477,17 @@
       <c r="K45" s="45"/>
       <c r="L45" s="45"/>
       <c r="M45" s="45"/>
-      <c r="N45" s="84" t="s">
+      <c r="N45" s="83" t="s">
         <v>5</v>
       </c>
-      <c r="O45" s="85"/>
-      <c r="P45" s="85"/>
+      <c r="O45" s="84"/>
+      <c r="P45" s="84"/>
       <c r="Q45" s="48">
         <f>SUM(Q10:Q44)</f>
-        <v>78.291200000000003</v>
-      </c>
-      <c r="R45" s="80"/>
-      <c r="S45" s="81"/>
+        <v>68.622200000000007</v>
+      </c>
+      <c r="R45" s="79"/>
+      <c r="S45" s="80"/>
     </row>
     <row r="46" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
@@ -6423,17 +6503,2343 @@
       <c r="K46" s="10"/>
       <c r="L46" s="10"/>
       <c r="M46" s="10"/>
-      <c r="N46" s="84" t="s">
+      <c r="N46" s="83" t="s">
         <v>6</v>
       </c>
-      <c r="O46" s="85"/>
-      <c r="P46" s="85"/>
+      <c r="O46" s="84"/>
+      <c r="P46" s="84"/>
       <c r="Q46" s="49">
         <f>Q45/10</f>
-        <v>7.8291200000000005</v>
-      </c>
-      <c r="R46" s="82"/>
-      <c r="S46" s="83"/>
+        <v>6.8622200000000007</v>
+      </c>
+      <c r="R46" s="81"/>
+      <c r="S46" s="82"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="K1:S1"/>
+    <mergeCell ref="S3:S8"/>
+    <mergeCell ref="N45:P45"/>
+    <mergeCell ref="R45:S46"/>
+    <mergeCell ref="N46:P46"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="O10" r:id="rId1"/>
+    <hyperlink ref="O11" r:id="rId2"/>
+    <hyperlink ref="O12" r:id="rId3"/>
+    <hyperlink ref="O13" r:id="rId4"/>
+    <hyperlink ref="O14" r:id="rId5"/>
+    <hyperlink ref="O15" r:id="rId6"/>
+    <hyperlink ref="O16" r:id="rId7"/>
+    <hyperlink ref="O17" r:id="rId8"/>
+    <hyperlink ref="O18" r:id="rId9"/>
+    <hyperlink ref="O19" r:id="rId10"/>
+    <hyperlink ref="O20" r:id="rId11"/>
+    <hyperlink ref="O21" r:id="rId12"/>
+    <hyperlink ref="O22" r:id="rId13"/>
+    <hyperlink ref="O27" r:id="rId14"/>
+    <hyperlink ref="O28" r:id="rId15"/>
+    <hyperlink ref="O30" r:id="rId16"/>
+    <hyperlink ref="O31" r:id="rId17"/>
+    <hyperlink ref="O32" r:id="rId18"/>
+    <hyperlink ref="O33" r:id="rId19"/>
+    <hyperlink ref="O34" r:id="rId20"/>
+    <hyperlink ref="O35" r:id="rId21"/>
+    <hyperlink ref="O37" r:id="rId22"/>
+    <hyperlink ref="O40" r:id="rId23"/>
+    <hyperlink ref="O24" r:id="rId24"/>
+    <hyperlink ref="O29" r:id="rId25"/>
+    <hyperlink ref="O36" r:id="rId26"/>
+    <hyperlink ref="O26" r:id="rId27"/>
+    <hyperlink ref="O41" r:id="rId28"/>
+    <hyperlink ref="O42" r:id="rId29"/>
+    <hyperlink ref="O43" r:id="rId30"/>
+    <hyperlink ref="O44" r:id="rId31"/>
+    <hyperlink ref="O39" r:id="rId32"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId33"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S46"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.28515625" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="26.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="75"/>
+      <c r="L1" s="75"/>
+      <c r="M1" s="75"/>
+      <c r="N1" s="75"/>
+      <c r="O1" s="75"/>
+      <c r="P1" s="75"/>
+      <c r="Q1" s="75"/>
+      <c r="R1" s="75"/>
+      <c r="S1" s="76"/>
+    </row>
+    <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="11"/>
+      <c r="F2" s="55" t="s">
+        <v>186</v>
+      </c>
+      <c r="G2" s="12"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="3"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="13"/>
+      <c r="F3" s="56" t="s">
+        <v>187</v>
+      </c>
+      <c r="G3" s="13"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
+      <c r="S3" s="77"/>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="13"/>
+      <c r="F4" s="57" t="s">
+        <v>187</v>
+      </c>
+      <c r="G4" s="14"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="78"/>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="F5" s="58" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="15"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="78"/>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="78"/>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="78"/>
+    </row>
+    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="78"/>
+    </row>
+    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="F9" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>106</v>
+      </c>
+      <c r="H9" s="30" t="s">
+        <v>132</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>189</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>148</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>185</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>231</v>
+      </c>
+      <c r="N9" s="30" t="s">
+        <v>232</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="P9" s="30" t="s">
+        <v>233</v>
+      </c>
+      <c r="Q9" s="30" t="s">
+        <v>234</v>
+      </c>
+      <c r="R9" s="30" t="s">
+        <v>196</v>
+      </c>
+      <c r="S9" s="30" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="69"/>
+      <c r="B10" s="46">
+        <f>ROW(B10) - ROW($B$9)</f>
+        <v>1</v>
+      </c>
+      <c r="C10" s="53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="G10" s="37" t="s">
+        <v>107</v>
+      </c>
+      <c r="H10" s="37" t="s">
+        <v>133</v>
+      </c>
+      <c r="I10" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J10" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="K10" s="37" t="s">
+        <v>171</v>
+      </c>
+      <c r="L10" s="37">
+        <v>1</v>
+      </c>
+      <c r="M10" s="37">
+        <f>L10*100</f>
+        <v>100</v>
+      </c>
+      <c r="N10" s="37">
+        <v>110</v>
+      </c>
+      <c r="O10" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P10" s="38">
+        <v>3.0530000000000002E-2</v>
+      </c>
+      <c r="Q10" s="38">
+        <f>P10*N10</f>
+        <v>3.3583000000000003</v>
+      </c>
+      <c r="R10" s="37"/>
+      <c r="S10" s="70"/>
+    </row>
+    <row r="11" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="69"/>
+      <c r="B11" s="47">
+        <f t="shared" ref="B11:B39" si="0">ROW(B11) - ROW($B$9)</f>
+        <v>2</v>
+      </c>
+      <c r="C11" s="53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="51" t="s">
+        <v>53</v>
+      </c>
+      <c r="F11" s="51" t="s">
+        <v>83</v>
+      </c>
+      <c r="G11" s="61" t="s">
+        <v>108</v>
+      </c>
+      <c r="H11" s="51" t="s">
+        <v>134</v>
+      </c>
+      <c r="I11" s="51" t="s">
+        <v>201</v>
+      </c>
+      <c r="J11" s="51" t="s">
+        <v>202</v>
+      </c>
+      <c r="K11" s="51" t="s">
+        <v>172</v>
+      </c>
+      <c r="L11" s="51">
+        <v>1</v>
+      </c>
+      <c r="M11" s="37">
+        <f t="shared" ref="M11:M44" si="1">L11*100</f>
+        <v>100</v>
+      </c>
+      <c r="N11" s="51">
+        <v>150</v>
+      </c>
+      <c r="O11" s="62" t="s">
+        <v>200</v>
+      </c>
+      <c r="P11" s="52">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="Q11" s="52">
+        <f t="shared" ref="Q11" si="2">P11*N11</f>
+        <v>1.05</v>
+      </c>
+      <c r="R11" s="51"/>
+      <c r="S11" s="51"/>
+    </row>
+    <row r="12" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="69"/>
+      <c r="B12" s="46">
+        <f>ROW(B12) - ROW($B$9)</f>
+        <v>3</v>
+      </c>
+      <c r="C12" s="53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="37" t="s">
+        <v>54</v>
+      </c>
+      <c r="F12" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="G12" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="H12" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="I12" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J12" s="37" t="s">
+        <v>150</v>
+      </c>
+      <c r="K12" s="37" t="s">
+        <v>171</v>
+      </c>
+      <c r="L12" s="37">
+        <v>7</v>
+      </c>
+      <c r="M12" s="37">
+        <f t="shared" si="1"/>
+        <v>700</v>
+      </c>
+      <c r="N12" s="37">
+        <v>800</v>
+      </c>
+      <c r="O12" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P12" s="38">
+        <v>6.4999999999999997E-3</v>
+      </c>
+      <c r="Q12" s="38">
+        <f>P12*N12</f>
+        <v>5.2</v>
+      </c>
+      <c r="R12" s="37"/>
+      <c r="S12" s="59"/>
+    </row>
+    <row r="13" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="69"/>
+      <c r="B13" s="47">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C13" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="51" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="51" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" s="51" t="s">
+        <v>85</v>
+      </c>
+      <c r="G13" s="51" t="s">
+        <v>110</v>
+      </c>
+      <c r="H13" s="51" t="s">
+        <v>133</v>
+      </c>
+      <c r="I13" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="J13" s="51" t="s">
+        <v>151</v>
+      </c>
+      <c r="K13" s="51" t="s">
+        <v>173</v>
+      </c>
+      <c r="L13" s="51">
+        <v>1</v>
+      </c>
+      <c r="M13" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N13" s="51">
+        <v>120</v>
+      </c>
+      <c r="O13" s="62" t="s">
+        <v>200</v>
+      </c>
+      <c r="P13" s="52">
+        <v>2.7799999999999998E-2</v>
+      </c>
+      <c r="Q13" s="52">
+        <f t="shared" ref="Q13" si="3">P13*N13</f>
+        <v>3.3359999999999999</v>
+      </c>
+      <c r="R13" s="51"/>
+      <c r="S13" s="59"/>
+    </row>
+    <row r="14" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A14" s="69"/>
+      <c r="B14" s="46">
+        <f>ROW(B14) - ROW($B$9)</f>
+        <v>5</v>
+      </c>
+      <c r="C14" s="53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="F14" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="G14" s="37" t="s">
+        <v>111</v>
+      </c>
+      <c r="H14" s="37" t="s">
+        <v>135</v>
+      </c>
+      <c r="I14" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J14" s="37" t="s">
+        <v>152</v>
+      </c>
+      <c r="K14" s="37" t="s">
+        <v>174</v>
+      </c>
+      <c r="L14" s="37">
+        <v>1</v>
+      </c>
+      <c r="M14" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N14" s="37">
+        <v>150</v>
+      </c>
+      <c r="O14" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P14" s="38">
+        <v>9.2999999999999992E-3</v>
+      </c>
+      <c r="Q14" s="38">
+        <f>P14*N14</f>
+        <v>1.3949999999999998</v>
+      </c>
+      <c r="R14" s="37"/>
+      <c r="S14" s="59"/>
+    </row>
+    <row r="15" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A15" s="69"/>
+      <c r="B15" s="47">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C15" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="51" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15" s="51" t="s">
+        <v>57</v>
+      </c>
+      <c r="F15" s="51" t="s">
+        <v>86</v>
+      </c>
+      <c r="G15" s="51" t="s">
+        <v>112</v>
+      </c>
+      <c r="H15" s="51" t="s">
+        <v>133</v>
+      </c>
+      <c r="I15" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="J15" s="51" t="s">
+        <v>153</v>
+      </c>
+      <c r="K15" s="51" t="s">
+        <v>175</v>
+      </c>
+      <c r="L15" s="51">
+        <v>1</v>
+      </c>
+      <c r="M15" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N15" s="51">
+        <v>120</v>
+      </c>
+      <c r="O15" s="62" t="s">
+        <v>200</v>
+      </c>
+      <c r="P15" s="52">
+        <v>1.9800000000000002E-2</v>
+      </c>
+      <c r="Q15" s="52">
+        <f t="shared" ref="Q15" si="4">P15*N15</f>
+        <v>2.3760000000000003</v>
+      </c>
+      <c r="R15" s="51"/>
+      <c r="S15" s="59"/>
+    </row>
+    <row r="16" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="69"/>
+      <c r="B16" s="46">
+        <f>ROW(B16) - ROW($B$9)</f>
+        <v>7</v>
+      </c>
+      <c r="C16" s="53" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="G16" s="37" t="s">
+        <v>113</v>
+      </c>
+      <c r="H16" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="I16" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J16" s="37" t="s">
+        <v>154</v>
+      </c>
+      <c r="K16" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="L16" s="37">
+        <v>7</v>
+      </c>
+      <c r="M16" s="37">
+        <f t="shared" si="1"/>
+        <v>700</v>
+      </c>
+      <c r="N16" s="37">
+        <v>800</v>
+      </c>
+      <c r="O16" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P16" s="38">
+        <v>5.8999999999999999E-3</v>
+      </c>
+      <c r="Q16" s="38">
+        <f>P16*N16</f>
+        <v>4.72</v>
+      </c>
+      <c r="R16" s="37"/>
+      <c r="S16" s="59"/>
+    </row>
+    <row r="17" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="69"/>
+      <c r="B17" s="47">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="C17" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" s="51" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" s="51" t="s">
+        <v>59</v>
+      </c>
+      <c r="F17" s="51" t="s">
+        <v>86</v>
+      </c>
+      <c r="G17" s="51" t="s">
+        <v>114</v>
+      </c>
+      <c r="H17" s="51" t="s">
+        <v>137</v>
+      </c>
+      <c r="I17" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="J17" s="51" t="s">
+        <v>155</v>
+      </c>
+      <c r="K17" s="51" t="s">
+        <v>176</v>
+      </c>
+      <c r="L17" s="51">
+        <v>1</v>
+      </c>
+      <c r="M17" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N17" s="51">
+        <v>150</v>
+      </c>
+      <c r="O17" s="62" t="s">
+        <v>200</v>
+      </c>
+      <c r="P17" s="52">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="Q17" s="52">
+        <f t="shared" ref="Q17" si="5">P17*N17</f>
+        <v>0.46499999999999997</v>
+      </c>
+      <c r="R17" s="51"/>
+      <c r="S17" s="59"/>
+    </row>
+    <row r="18" spans="1:19" s="71" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A18" s="69"/>
+      <c r="B18" s="46">
+        <f>ROW(B18) - ROW($B$9)</f>
+        <v>9</v>
+      </c>
+      <c r="C18" s="53" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="F18" s="37" t="s">
+        <v>199</v>
+      </c>
+      <c r="G18" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="H18" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="I18" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J18" s="37" t="s">
+        <v>156</v>
+      </c>
+      <c r="K18" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="L18" s="37">
+        <v>3</v>
+      </c>
+      <c r="M18" s="37">
+        <f t="shared" si="1"/>
+        <v>300</v>
+      </c>
+      <c r="N18" s="37">
+        <v>320</v>
+      </c>
+      <c r="O18" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P18" s="38">
+        <v>2.2100000000000002E-2</v>
+      </c>
+      <c r="Q18" s="38">
+        <f>P18*N18</f>
+        <v>7.072000000000001</v>
+      </c>
+      <c r="R18" s="37"/>
+      <c r="S18" s="59"/>
+    </row>
+    <row r="19" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A19" s="69"/>
+      <c r="B19" s="47">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="C19" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="51" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" s="51" t="s">
+        <v>61</v>
+      </c>
+      <c r="F19" s="51" t="s">
+        <v>199</v>
+      </c>
+      <c r="G19" s="51" t="s">
+        <v>89</v>
+      </c>
+      <c r="H19" s="51" t="s">
+        <v>139</v>
+      </c>
+      <c r="I19" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="J19" s="51" t="s">
+        <v>157</v>
+      </c>
+      <c r="K19" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="L19" s="51">
+        <v>1</v>
+      </c>
+      <c r="M19" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N19" s="51">
+        <v>105</v>
+      </c>
+      <c r="O19" s="62" t="s">
+        <v>200</v>
+      </c>
+      <c r="P19" s="52">
+        <v>0.17630000000000001</v>
+      </c>
+      <c r="Q19" s="52">
+        <f t="shared" ref="Q19" si="6">P19*N19</f>
+        <v>18.511500000000002</v>
+      </c>
+      <c r="R19" s="51"/>
+      <c r="S19" s="59"/>
+    </row>
+    <row r="20" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A20" s="69"/>
+      <c r="B20" s="46">
+        <f>ROW(B20) - ROW($B$9)</f>
+        <v>11</v>
+      </c>
+      <c r="C20" s="53" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="F20" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="G20" s="37" t="s">
+        <v>115</v>
+      </c>
+      <c r="H20" s="37" t="s">
+        <v>140</v>
+      </c>
+      <c r="I20" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J20" s="37" t="s">
+        <v>158</v>
+      </c>
+      <c r="K20" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="L20" s="37">
+        <v>2</v>
+      </c>
+      <c r="M20" s="37">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N20" s="37">
+        <v>250</v>
+      </c>
+      <c r="O20" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P20" s="38">
+        <v>1.21E-2</v>
+      </c>
+      <c r="Q20" s="38">
+        <f>P20*N20</f>
+        <v>3.0249999999999999</v>
+      </c>
+      <c r="R20" s="37"/>
+      <c r="S20" s="59"/>
+    </row>
+    <row r="21" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="69"/>
+      <c r="B21" s="47">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="C21" s="54" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="51" t="s">
+        <v>31</v>
+      </c>
+      <c r="E21" s="51" t="s">
+        <v>63</v>
+      </c>
+      <c r="F21" s="51" t="s">
+        <v>91</v>
+      </c>
+      <c r="G21" s="51" t="s">
+        <v>116</v>
+      </c>
+      <c r="H21" s="51" t="s">
+        <v>141</v>
+      </c>
+      <c r="I21" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="J21" s="51" t="s">
+        <v>159</v>
+      </c>
+      <c r="K21" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="L21" s="51">
+        <v>1</v>
+      </c>
+      <c r="M21" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N21" s="51">
+        <v>105</v>
+      </c>
+      <c r="O21" s="62" t="s">
+        <v>200</v>
+      </c>
+      <c r="P21" s="52">
+        <v>6.0299999999999999E-2</v>
+      </c>
+      <c r="Q21" s="52">
+        <f t="shared" ref="Q21" si="7">P21*N21</f>
+        <v>6.3315000000000001</v>
+      </c>
+      <c r="R21" s="51"/>
+      <c r="S21" s="59"/>
+    </row>
+    <row r="22" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A22" s="69"/>
+      <c r="B22" s="46">
+        <f>ROW(B22) - ROW($B$9)</f>
+        <v>13</v>
+      </c>
+      <c r="C22" s="53" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>64</v>
+      </c>
+      <c r="F22" s="37" t="s">
+        <v>203</v>
+      </c>
+      <c r="G22" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="H22" s="37" t="s">
+        <v>142</v>
+      </c>
+      <c r="I22" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J22" s="37" t="s">
+        <v>160</v>
+      </c>
+      <c r="K22" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="L22" s="37">
+        <v>1</v>
+      </c>
+      <c r="M22" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N22" s="37">
+        <v>105</v>
+      </c>
+      <c r="O22" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P22" s="38">
+        <v>0.1487</v>
+      </c>
+      <c r="Q22" s="38">
+        <f>P22*N22</f>
+        <v>15.6135</v>
+      </c>
+      <c r="R22" s="37"/>
+      <c r="S22" s="59"/>
+    </row>
+    <row r="23" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A23" s="69"/>
+      <c r="B23" s="47">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="C23" s="54" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="61" t="s">
+        <v>33</v>
+      </c>
+      <c r="E23" s="61" t="s">
+        <v>65</v>
+      </c>
+      <c r="F23" s="61" t="s">
+        <v>199</v>
+      </c>
+      <c r="G23" s="61" t="s">
+        <v>93</v>
+      </c>
+      <c r="H23" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="I23" s="61"/>
+      <c r="J23" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="K23" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="L23" s="61">
+        <v>6</v>
+      </c>
+      <c r="M23" s="61">
+        <f t="shared" si="1"/>
+        <v>600</v>
+      </c>
+      <c r="N23" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="O23" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="P23" s="72" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q23" s="72" t="s">
+        <v>198</v>
+      </c>
+      <c r="R23" s="73" t="s">
+        <v>214</v>
+      </c>
+      <c r="S23" s="65"/>
+    </row>
+    <row r="24" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A24" s="69"/>
+      <c r="B24" s="46">
+        <f>ROW(B24) - ROW($B$9)</f>
+        <v>15</v>
+      </c>
+      <c r="C24" s="53" t="s">
+        <v>188</v>
+      </c>
+      <c r="D24" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="E24" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="F24" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="G24" s="68" t="s">
+        <v>117</v>
+      </c>
+      <c r="H24" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="I24" s="37" t="s">
+        <v>204</v>
+      </c>
+      <c r="J24" s="37" t="s">
+        <v>205</v>
+      </c>
+      <c r="K24" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="L24" s="37">
+        <v>1</v>
+      </c>
+      <c r="M24" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N24" s="37">
+        <v>200</v>
+      </c>
+      <c r="O24" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P24" s="38">
+        <v>5.8999999999999999E-3</v>
+      </c>
+      <c r="Q24" s="38">
+        <f>P24*N24</f>
+        <v>1.18</v>
+      </c>
+      <c r="R24" s="37"/>
+      <c r="S24" s="59"/>
+    </row>
+    <row r="25" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A25" s="69"/>
+      <c r="B25" s="47">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C25" s="54" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="61" t="s">
+        <v>35</v>
+      </c>
+      <c r="E25" s="61" t="s">
+        <v>65</v>
+      </c>
+      <c r="F25" s="61" t="s">
+        <v>199</v>
+      </c>
+      <c r="G25" s="61" t="s">
+        <v>95</v>
+      </c>
+      <c r="H25" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="I25" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="J25" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="K25" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="L25" s="61">
+        <v>1</v>
+      </c>
+      <c r="M25" s="61">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N25" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="O25" s="61" t="s">
+        <v>198</v>
+      </c>
+      <c r="P25" s="72" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q25" s="72" t="s">
+        <v>198</v>
+      </c>
+      <c r="R25" s="73" t="s">
+        <v>214</v>
+      </c>
+      <c r="S25" s="65"/>
+    </row>
+    <row r="26" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="69"/>
+      <c r="B26" s="46">
+        <f>ROW(B26) - ROW($B$9)</f>
+        <v>17</v>
+      </c>
+      <c r="C26" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="E26" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="F26" s="37" t="s">
+        <v>96</v>
+      </c>
+      <c r="G26" s="68" t="s">
+        <v>118</v>
+      </c>
+      <c r="H26" s="37" t="s">
+        <v>144</v>
+      </c>
+      <c r="I26" s="37" t="s">
+        <v>215</v>
+      </c>
+      <c r="J26" s="37" t="s">
+        <v>209</v>
+      </c>
+      <c r="K26" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="L26" s="37">
+        <v>2</v>
+      </c>
+      <c r="M26" s="37">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N26" s="37">
+        <v>202</v>
+      </c>
+      <c r="O26" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P26" s="38">
+        <v>0.65390000000000004</v>
+      </c>
+      <c r="Q26" s="38">
+        <f>P26*N26</f>
+        <v>132.08780000000002</v>
+      </c>
+      <c r="R26" s="37"/>
+      <c r="S26" s="59"/>
+    </row>
+    <row r="27" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A27" s="69"/>
+      <c r="B27" s="47">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="C27" s="54" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" s="51" t="s">
+        <v>37</v>
+      </c>
+      <c r="E27" s="51" t="s">
+        <v>68</v>
+      </c>
+      <c r="F27" s="51" t="s">
+        <v>97</v>
+      </c>
+      <c r="G27" s="51" t="s">
+        <v>119</v>
+      </c>
+      <c r="H27" s="51" t="s">
+        <v>140</v>
+      </c>
+      <c r="I27" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="J27" s="51" t="s">
+        <v>161</v>
+      </c>
+      <c r="K27" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="L27" s="51">
+        <v>1</v>
+      </c>
+      <c r="M27" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N27" s="51">
+        <v>110</v>
+      </c>
+      <c r="O27" s="62" t="s">
+        <v>200</v>
+      </c>
+      <c r="P27" s="52">
+        <v>3.1699999999999999E-2</v>
+      </c>
+      <c r="Q27" s="52">
+        <f t="shared" ref="Q27" si="8">P27*N27</f>
+        <v>3.4870000000000001</v>
+      </c>
+      <c r="R27" s="51"/>
+      <c r="S27" s="59"/>
+    </row>
+    <row r="28" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A28" s="69"/>
+      <c r="B28" s="46">
+        <f>ROW(B28) - ROW($B$9)</f>
+        <v>19</v>
+      </c>
+      <c r="C28" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="E28" s="37" t="s">
+        <v>69</v>
+      </c>
+      <c r="F28" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="G28" s="37" t="s">
+        <v>120</v>
+      </c>
+      <c r="H28" s="37" t="s">
+        <v>133</v>
+      </c>
+      <c r="I28" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J28" s="37" t="s">
+        <v>162</v>
+      </c>
+      <c r="K28" s="37" t="s">
+        <v>177</v>
+      </c>
+      <c r="L28" s="37">
+        <v>9</v>
+      </c>
+      <c r="M28" s="37">
+        <f t="shared" si="1"/>
+        <v>900</v>
+      </c>
+      <c r="N28" s="37">
+        <v>1000</v>
+      </c>
+      <c r="O28" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P28" s="38">
+        <v>3.3E-3</v>
+      </c>
+      <c r="Q28" s="38">
+        <f>P28*N28</f>
+        <v>3.3</v>
+      </c>
+      <c r="R28" s="51"/>
+      <c r="S28" s="59"/>
+    </row>
+    <row r="29" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="69"/>
+      <c r="B29" s="47">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="C29" s="54" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" s="51" t="s">
+        <v>39</v>
+      </c>
+      <c r="E29" s="51" t="s">
+        <v>70</v>
+      </c>
+      <c r="F29" s="51" t="s">
+        <v>98</v>
+      </c>
+      <c r="G29" s="61" t="s">
+        <v>121</v>
+      </c>
+      <c r="H29" s="51" t="s">
+        <v>133</v>
+      </c>
+      <c r="I29" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="J29" s="51" t="s">
+        <v>206</v>
+      </c>
+      <c r="K29" s="51" t="s">
+        <v>178</v>
+      </c>
+      <c r="L29" s="51">
+        <v>1</v>
+      </c>
+      <c r="M29" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N29" s="51">
+        <v>200</v>
+      </c>
+      <c r="O29" s="62" t="s">
+        <v>200</v>
+      </c>
+      <c r="P29" s="52">
+        <v>1.4E-3</v>
+      </c>
+      <c r="Q29" s="52">
+        <f t="shared" ref="Q29" si="9">P29*N29</f>
+        <v>0.27999999999999997</v>
+      </c>
+      <c r="R29" s="51"/>
+      <c r="S29" s="59"/>
+    </row>
+    <row r="30" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="69"/>
+      <c r="B30" s="46">
+        <f>ROW(B30) - ROW($B$9)</f>
+        <v>21</v>
+      </c>
+      <c r="C30" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="D30" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="E30" s="37" t="s">
+        <v>71</v>
+      </c>
+      <c r="F30" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="G30" s="37" t="s">
+        <v>122</v>
+      </c>
+      <c r="H30" s="37" t="s">
+        <v>133</v>
+      </c>
+      <c r="I30" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J30" s="37" t="s">
+        <v>163</v>
+      </c>
+      <c r="K30" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="L30" s="37">
+        <v>5</v>
+      </c>
+      <c r="M30" s="37">
+        <f t="shared" si="1"/>
+        <v>500</v>
+      </c>
+      <c r="N30" s="37">
+        <v>600</v>
+      </c>
+      <c r="O30" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P30" s="38">
+        <v>6.9999999999999999E-4</v>
+      </c>
+      <c r="Q30" s="38">
+        <f>P30*N30</f>
+        <v>0.42</v>
+      </c>
+      <c r="R30" s="37"/>
+      <c r="S30" s="59"/>
+    </row>
+    <row r="31" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A31" s="69"/>
+      <c r="B31" s="47">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="C31" s="54" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" s="51" t="s">
+        <v>41</v>
+      </c>
+      <c r="E31" s="51" t="s">
+        <v>72</v>
+      </c>
+      <c r="F31" s="51" t="s">
+        <v>100</v>
+      </c>
+      <c r="G31" s="51" t="s">
+        <v>123</v>
+      </c>
+      <c r="H31" s="51" t="s">
+        <v>145</v>
+      </c>
+      <c r="I31" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="J31" s="51" t="s">
+        <v>164</v>
+      </c>
+      <c r="K31" s="51" t="s">
+        <v>180</v>
+      </c>
+      <c r="L31" s="51">
+        <v>1</v>
+      </c>
+      <c r="M31" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N31" s="51">
+        <v>105</v>
+      </c>
+      <c r="O31" s="62" t="s">
+        <v>200</v>
+      </c>
+      <c r="P31" s="52">
+        <v>0.16569999999999999</v>
+      </c>
+      <c r="Q31" s="52">
+        <f t="shared" ref="Q31" si="10">P31*N31</f>
+        <v>17.398499999999999</v>
+      </c>
+      <c r="R31" s="51"/>
+      <c r="S31" s="59"/>
+    </row>
+    <row r="32" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="69"/>
+      <c r="B32" s="46">
+        <f>ROW(B32) - ROW($B$9)</f>
+        <v>23</v>
+      </c>
+      <c r="C32" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="D32" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="E32" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="F32" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="G32" s="37" t="s">
+        <v>124</v>
+      </c>
+      <c r="H32" s="37" t="s">
+        <v>133</v>
+      </c>
+      <c r="I32" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J32" s="37" t="s">
+        <v>165</v>
+      </c>
+      <c r="K32" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="L32" s="37">
+        <v>1</v>
+      </c>
+      <c r="M32" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N32" s="37">
+        <v>200</v>
+      </c>
+      <c r="O32" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P32" s="38">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="Q32" s="38">
+        <f>P32*N32</f>
+        <v>0.12</v>
+      </c>
+      <c r="R32" s="37"/>
+      <c r="S32" s="59"/>
+    </row>
+    <row r="33" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="69"/>
+      <c r="B33" s="47">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="C33" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="D33" s="51" t="s">
+        <v>43</v>
+      </c>
+      <c r="E33" s="51" t="s">
+        <v>74</v>
+      </c>
+      <c r="F33" s="51" t="s">
+        <v>99</v>
+      </c>
+      <c r="G33" s="51" t="s">
+        <v>125</v>
+      </c>
+      <c r="H33" s="51" t="s">
+        <v>133</v>
+      </c>
+      <c r="I33" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="J33" s="51" t="s">
+        <v>166</v>
+      </c>
+      <c r="K33" s="51" t="s">
+        <v>181</v>
+      </c>
+      <c r="L33" s="51">
+        <v>1</v>
+      </c>
+      <c r="M33" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N33" s="51">
+        <v>200</v>
+      </c>
+      <c r="O33" s="62" t="s">
+        <v>200</v>
+      </c>
+      <c r="P33" s="52">
+        <v>6.9999999999999999E-4</v>
+      </c>
+      <c r="Q33" s="52">
+        <f t="shared" ref="Q33" si="11">P33*N33</f>
+        <v>0.13999999999999999</v>
+      </c>
+      <c r="R33" s="51"/>
+      <c r="S33" s="59"/>
+    </row>
+    <row r="34" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="69"/>
+      <c r="B34" s="46">
+        <f>ROW(B34) - ROW($B$9)</f>
+        <v>25</v>
+      </c>
+      <c r="C34" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="D34" s="37" t="s">
+        <v>44</v>
+      </c>
+      <c r="E34" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="F34" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="G34" s="37" t="s">
+        <v>126</v>
+      </c>
+      <c r="H34" s="37" t="s">
+        <v>133</v>
+      </c>
+      <c r="I34" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J34" s="37" t="s">
+        <v>167</v>
+      </c>
+      <c r="K34" s="37" t="s">
+        <v>182</v>
+      </c>
+      <c r="L34" s="37">
+        <v>1</v>
+      </c>
+      <c r="M34" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N34" s="37">
+        <v>200</v>
+      </c>
+      <c r="O34" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P34" s="38">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="Q34" s="38">
+        <f>P34*N34</f>
+        <v>0.44</v>
+      </c>
+      <c r="R34" s="37"/>
+      <c r="S34" s="59"/>
+    </row>
+    <row r="35" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="69"/>
+      <c r="B35" s="47">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="C35" s="54" t="s">
+        <v>16</v>
+      </c>
+      <c r="D35" s="51" t="s">
+        <v>45</v>
+      </c>
+      <c r="E35" s="51" t="s">
+        <v>76</v>
+      </c>
+      <c r="F35" s="51" t="s">
+        <v>98</v>
+      </c>
+      <c r="G35" s="51" t="s">
+        <v>127</v>
+      </c>
+      <c r="H35" s="51" t="s">
+        <v>133</v>
+      </c>
+      <c r="I35" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="J35" s="51" t="s">
+        <v>168</v>
+      </c>
+      <c r="K35" s="51" t="s">
+        <v>183</v>
+      </c>
+      <c r="L35" s="51">
+        <v>3</v>
+      </c>
+      <c r="M35" s="37">
+        <f t="shared" si="1"/>
+        <v>300</v>
+      </c>
+      <c r="N35" s="51">
+        <v>400</v>
+      </c>
+      <c r="O35" s="62" t="s">
+        <v>200</v>
+      </c>
+      <c r="P35" s="52">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="Q35" s="52">
+        <f t="shared" ref="Q35" si="12">P35*N35</f>
+        <v>0.88</v>
+      </c>
+      <c r="R35" s="51"/>
+      <c r="S35" s="59"/>
+    </row>
+    <row r="36" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="69"/>
+      <c r="B36" s="46">
+        <f>ROW(B36) - ROW($B$9)</f>
+        <v>27</v>
+      </c>
+      <c r="C36" s="53" t="s">
+        <v>16</v>
+      </c>
+      <c r="D36" s="37" t="s">
+        <v>46</v>
+      </c>
+      <c r="E36" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="F36" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="G36" s="68" t="s">
+        <v>128</v>
+      </c>
+      <c r="H36" s="37" t="s">
+        <v>133</v>
+      </c>
+      <c r="I36" s="37" t="s">
+        <v>207</v>
+      </c>
+      <c r="J36" s="37" t="s">
+        <v>208</v>
+      </c>
+      <c r="K36" s="37" t="s">
+        <v>184</v>
+      </c>
+      <c r="L36" s="37">
+        <v>1</v>
+      </c>
+      <c r="M36" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N36" s="37">
+        <v>200</v>
+      </c>
+      <c r="O36" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P36" s="38">
+        <v>1.6999999999999999E-3</v>
+      </c>
+      <c r="Q36" s="38">
+        <f>P36*N36</f>
+        <v>0.33999999999999997</v>
+      </c>
+      <c r="R36" s="37"/>
+      <c r="S36" s="59"/>
+    </row>
+    <row r="37" spans="1:19" s="71" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="69"/>
+      <c r="B37" s="47">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="C37" s="54" t="s">
+        <v>16</v>
+      </c>
+      <c r="D37" s="51" t="s">
+        <v>47</v>
+      </c>
+      <c r="E37" s="51" t="s">
+        <v>78</v>
+      </c>
+      <c r="F37" s="51" t="s">
+        <v>102</v>
+      </c>
+      <c r="G37" s="51" t="s">
+        <v>129</v>
+      </c>
+      <c r="H37" s="51" t="s">
+        <v>133</v>
+      </c>
+      <c r="I37" s="51" t="s">
+        <v>198</v>
+      </c>
+      <c r="J37" s="51" t="s">
+        <v>169</v>
+      </c>
+      <c r="K37" s="51" t="s">
+        <v>179</v>
+      </c>
+      <c r="L37" s="51">
+        <v>4</v>
+      </c>
+      <c r="M37" s="37">
+        <f t="shared" si="1"/>
+        <v>400</v>
+      </c>
+      <c r="N37" s="51">
+        <v>500</v>
+      </c>
+      <c r="O37" s="62" t="s">
+        <v>200</v>
+      </c>
+      <c r="P37" s="52">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="Q37" s="52">
+        <f t="shared" ref="Q37" si="13">P37*N37</f>
+        <v>0.45</v>
+      </c>
+      <c r="R37" s="51"/>
+      <c r="S37" s="59"/>
+    </row>
+    <row r="38" spans="1:19" s="71" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A38" s="69"/>
+      <c r="B38" s="46">
+        <f>ROW(B38) - ROW($B$9)</f>
+        <v>29</v>
+      </c>
+      <c r="C38" s="53" t="s">
+        <v>17</v>
+      </c>
+      <c r="D38" s="68" t="s">
+        <v>48</v>
+      </c>
+      <c r="E38" s="68" t="s">
+        <v>79</v>
+      </c>
+      <c r="F38" s="68" t="s">
+        <v>199</v>
+      </c>
+      <c r="G38" s="68" t="s">
+        <v>103</v>
+      </c>
+      <c r="H38" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="I38" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="J38" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="K38" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="L38" s="68">
+        <v>7</v>
+      </c>
+      <c r="M38" s="68">
+        <f t="shared" si="1"/>
+        <v>700</v>
+      </c>
+      <c r="N38" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="O38" s="68" t="s">
+        <v>198</v>
+      </c>
+      <c r="P38" s="74" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q38" s="74" t="s">
+        <v>198</v>
+      </c>
+      <c r="R38" s="73" t="s">
+        <v>214</v>
+      </c>
+      <c r="S38" s="65"/>
+    </row>
+    <row r="39" spans="1:19" s="87" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="85"/>
+      <c r="B39" s="88">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="C39" s="93" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" s="89" t="s">
+        <v>49</v>
+      </c>
+      <c r="E39" s="89" t="s">
+        <v>80</v>
+      </c>
+      <c r="F39" s="89" t="s">
+        <v>104</v>
+      </c>
+      <c r="G39" s="89" t="s">
+        <v>130</v>
+      </c>
+      <c r="H39" s="89" t="s">
+        <v>146</v>
+      </c>
+      <c r="I39" s="89" t="s">
+        <v>198</v>
+      </c>
+      <c r="J39" s="89" t="s">
+        <v>198</v>
+      </c>
+      <c r="K39" s="89" t="s">
+        <v>198</v>
+      </c>
+      <c r="L39" s="89">
+        <v>1</v>
+      </c>
+      <c r="M39" s="86">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N39" s="89">
+        <v>101</v>
+      </c>
+      <c r="O39" s="90" t="s">
+        <v>235</v>
+      </c>
+      <c r="P39" s="91">
+        <v>1.4650000000000001</v>
+      </c>
+      <c r="Q39" s="91">
+        <f t="shared" ref="Q39" si="14">P39*N39</f>
+        <v>147.965</v>
+      </c>
+      <c r="R39" s="89"/>
+      <c r="S39" s="92"/>
+    </row>
+    <row r="40" spans="1:19" s="71" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="69"/>
+      <c r="B40" s="46">
+        <f>ROW(B40) - ROW($B$9)</f>
+        <v>31</v>
+      </c>
+      <c r="C40" s="53" t="s">
+        <v>18</v>
+      </c>
+      <c r="D40" s="37" t="s">
+        <v>50</v>
+      </c>
+      <c r="E40" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="F40" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="G40" s="37" t="s">
+        <v>131</v>
+      </c>
+      <c r="H40" s="37" t="s">
+        <v>147</v>
+      </c>
+      <c r="I40" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J40" s="37" t="s">
+        <v>170</v>
+      </c>
+      <c r="K40" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="L40" s="37">
+        <v>1</v>
+      </c>
+      <c r="M40" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N40" s="37">
+        <v>101</v>
+      </c>
+      <c r="O40" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P40" s="38">
+        <v>0.62890000000000001</v>
+      </c>
+      <c r="Q40" s="38">
+        <f>P40*N40</f>
+        <v>63.518900000000002</v>
+      </c>
+      <c r="R40" s="37"/>
+      <c r="S40" s="39"/>
+    </row>
+    <row r="41" spans="1:19" s="71" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="69"/>
+      <c r="B41" s="46">
+        <f t="shared" ref="B41:B44" si="15">ROW(B41) - ROW($B$9)</f>
+        <v>32</v>
+      </c>
+      <c r="C41" s="53" t="s">
+        <v>216</v>
+      </c>
+      <c r="D41" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="E41" s="37" t="s">
+        <v>218</v>
+      </c>
+      <c r="F41" s="37" t="s">
+        <v>199</v>
+      </c>
+      <c r="G41" s="37" t="s">
+        <v>217</v>
+      </c>
+      <c r="H41" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="I41" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J41" s="37" t="s">
+        <v>220</v>
+      </c>
+      <c r="K41" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="L41" s="37">
+        <v>1</v>
+      </c>
+      <c r="M41" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N41" s="37">
+        <v>100</v>
+      </c>
+      <c r="O41" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P41" s="38">
+        <v>9.3100000000000002E-2</v>
+      </c>
+      <c r="Q41" s="38">
+        <f>P41*N41</f>
+        <v>9.31</v>
+      </c>
+      <c r="R41" s="37"/>
+      <c r="S41" s="39"/>
+    </row>
+    <row r="42" spans="1:19" s="71" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="69"/>
+      <c r="B42" s="46">
+        <f t="shared" si="15"/>
+        <v>33</v>
+      </c>
+      <c r="C42" s="53" t="s">
+        <v>216</v>
+      </c>
+      <c r="D42" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="E42" s="37" t="s">
+        <v>223</v>
+      </c>
+      <c r="F42" s="37" t="s">
+        <v>199</v>
+      </c>
+      <c r="G42" s="37" t="s">
+        <v>221</v>
+      </c>
+      <c r="H42" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="I42" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J42" s="37" t="s">
+        <v>222</v>
+      </c>
+      <c r="K42" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="L42" s="37">
+        <v>1</v>
+      </c>
+      <c r="M42" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N42" s="37">
+        <v>100</v>
+      </c>
+      <c r="O42" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P42" s="38">
+        <v>5.16E-2</v>
+      </c>
+      <c r="Q42" s="38">
+        <f t="shared" ref="Q42:Q44" si="16">P42*N42</f>
+        <v>5.16</v>
+      </c>
+      <c r="R42" s="37"/>
+      <c r="S42" s="39"/>
+    </row>
+    <row r="43" spans="1:19" s="71" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="69"/>
+      <c r="B43" s="46">
+        <f t="shared" si="15"/>
+        <v>34</v>
+      </c>
+      <c r="C43" s="53" t="s">
+        <v>216</v>
+      </c>
+      <c r="D43" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="E43" s="37" t="s">
+        <v>224</v>
+      </c>
+      <c r="F43" s="37" t="s">
+        <v>199</v>
+      </c>
+      <c r="G43" s="37" t="s">
+        <v>225</v>
+      </c>
+      <c r="H43" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="I43" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J43" s="37" t="s">
+        <v>226</v>
+      </c>
+      <c r="K43" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="L43" s="37">
+        <v>2</v>
+      </c>
+      <c r="M43" s="37">
+        <f t="shared" si="1"/>
+        <v>200</v>
+      </c>
+      <c r="N43" s="37">
+        <v>200</v>
+      </c>
+      <c r="O43" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P43" s="38">
+        <v>5.9900000000000002E-2</v>
+      </c>
+      <c r="Q43" s="38">
+        <f t="shared" si="16"/>
+        <v>11.98</v>
+      </c>
+      <c r="R43" s="37"/>
+      <c r="S43" s="39"/>
+    </row>
+    <row r="44" spans="1:19" s="71" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="69"/>
+      <c r="B44" s="46">
+        <f t="shared" si="15"/>
+        <v>35</v>
+      </c>
+      <c r="C44" s="53" t="s">
+        <v>216</v>
+      </c>
+      <c r="D44" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="E44" s="37" t="s">
+        <v>229</v>
+      </c>
+      <c r="F44" s="37" t="s">
+        <v>199</v>
+      </c>
+      <c r="G44" s="37" t="s">
+        <v>227</v>
+      </c>
+      <c r="H44" s="37" t="s">
+        <v>228</v>
+      </c>
+      <c r="I44" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="J44" s="37" t="s">
+        <v>230</v>
+      </c>
+      <c r="K44" s="37" t="s">
+        <v>198</v>
+      </c>
+      <c r="L44" s="37">
+        <v>1</v>
+      </c>
+      <c r="M44" s="37">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+      <c r="N44" s="37">
+        <v>105</v>
+      </c>
+      <c r="O44" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="P44" s="38">
+        <v>6.8099999999999994E-2</v>
+      </c>
+      <c r="Q44" s="38">
+        <f t="shared" si="16"/>
+        <v>7.1504999999999992</v>
+      </c>
+      <c r="R44" s="37"/>
+      <c r="S44" s="39"/>
+    </row>
+    <row r="45" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="1"/>
+      <c r="B45" s="40"/>
+      <c r="C45" s="41"/>
+      <c r="D45" s="42"/>
+      <c r="E45" s="43"/>
+      <c r="F45" s="44"/>
+      <c r="G45" s="45"/>
+      <c r="H45" s="44"/>
+      <c r="I45" s="45"/>
+      <c r="J45" s="44"/>
+      <c r="K45" s="45"/>
+      <c r="L45" s="45"/>
+      <c r="M45" s="45"/>
+      <c r="N45" s="83" t="s">
+        <v>5</v>
+      </c>
+      <c r="O45" s="84"/>
+      <c r="P45" s="84"/>
+      <c r="Q45" s="48">
+        <f>SUM(Q10:Q44)</f>
+        <v>478.06150000000008</v>
+      </c>
+      <c r="R45" s="79"/>
+      <c r="S45" s="80"/>
+    </row>
+    <row r="46" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="1"/>
+      <c r="B46" s="25"/>
+      <c r="C46" s="36"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="10"/>
+      <c r="I46" s="10"/>
+      <c r="J46" s="10"/>
+      <c r="K46" s="10"/>
+      <c r="L46" s="10"/>
+      <c r="M46" s="10"/>
+      <c r="N46" s="83" t="s">
+        <v>6</v>
+      </c>
+      <c r="O46" s="84"/>
+      <c r="P46" s="84"/>
+      <c r="Q46" s="49">
+        <f>Q45/100</f>
+        <v>4.7806150000000009</v>
+      </c>
+      <c r="R46" s="81"/>
+      <c r="S46" s="82"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>